<commit_message>
Chỉnh báo cáo theo góp ý: chi tiết theo Ngày test, mục tiêu nhập tay, Tuần=Tháng
- Bảng chi tiết Trang/Tính năng: lấy từ 02_UI_UX & 03_Tính_năng theo Ngày test gần nhất
  trong kỳ (trạng thái Hoàn thành/Kiểm tra lại), kèm cột Số lỗi và Ngày test/retest.
- Cột Mục tiêu kỳ để trống cho BGD/Tester tự nhập; Tỷ lệ đạt = Kết quả/Mục tiêu.
- Gộp layout: sheet Tuần dùng chung bố cục với sheet Tháng, chỉ khác mốc lọc theo tuần.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013S9deAhjLT6GCCVgruMn8Z
</commit_message>
<xml_diff>
--- a/BaoCao_BGD_TimViec123.xlsx
+++ b/BaoCao_BGD_TimViec123.xlsx
@@ -4,22 +4,24 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="10" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="z_Config" sheetId="1" state="hidden" r:id="rId1"/>
     <sheet name="z_Trang" sheetId="2" state="hidden" r:id="rId2"/>
     <sheet name="z_TinhNang" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="z_Loi" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="z_CV" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="z_DB_DN" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="z_DB_HR" sheetId="7" state="hidden" r:id="rId7"/>
-    <sheet name="z_DB_UV" sheetId="8" state="hidden" r:id="rId8"/>
-    <sheet name="z_DB_Tin" sheetId="9" state="hidden" r:id="rId9"/>
-    <sheet name="00_Hướng_dẫn" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="01_Báo_cáo_Tháng" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="02_Báo_cáo_Tuần" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="03_Nghiệm_thu" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="z_TrangFull" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="z_TNFull" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="z_Loi" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="z_CV" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="z_DB_DN" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet name="z_DB_HR" sheetId="9" state="hidden" r:id="rId9"/>
+    <sheet name="z_DB_UV" sheetId="10" state="hidden" r:id="rId10"/>
+    <sheet name="z_DB_Tin" sheetId="11" state="hidden" r:id="rId11"/>
+    <sheet name="00_Hướng_dẫn" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="01_Báo_cáo_Tháng" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="02_Báo_cáo_Tuần" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="03_Nghiệm_thu" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +34,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,6 +133,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="10.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001A1A1A"/>
       <sz val="10.5"/>
     </font>
@@ -193,8 +201,8 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00B8860B"/>
-      <sz val="11"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -282,7 +290,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -354,7 +362,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -363,10 +371,10 @@
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -378,78 +386,78 @@
     <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="19" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -459,105 +467,100 @@
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="27" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="17" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="29" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="17" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="21" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="22" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -948,7 +951,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Năm báo cáo</t>
+          <t>Năm</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -975,11 +978,51 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>IMPORTRANGE('z_Config'!$B$3,"'HS ỨNG TUYỂN'!D5:D990")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1">
+        <f>IMPORTRANGE('z_Config'!$B$3,"'Tin tuyển dụng'!C4:D1006")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="001F3A5F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1052,7 +1095,7 @@
       <c r="B6" s="9" t="n"/>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Cập nhật dữ liệu tại file làm việc; báo cáo tự đồng bộ.</t>
+          <t>Cập nhật dữ liệu tại file làm việc; nhập Mục tiêu kỳ; báo cáo tự đồng bộ.</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1130,7 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Tiến độ trang = số trang Hoàn thành / tổng số trang (hiện 63).</t>
+          <t>Tiến độ trang = số trang Hoàn thành / tổng số trang (hiện 63). Tính năng / 88.</t>
         </is>
       </c>
       <c r="C10" s="14" t="n"/>
@@ -1101,7 +1144,7 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Tiến độ tính năng = số tính năng Hoàn thành / 88 tính năng (gồm YC_88 chờ flow).</t>
+          <t>Số lỗi lấy toàn bộ từ 05_Lỗi_Tester. "Đang mở" = Open + Chưa gửi Dev; "Đã xử lý" = Fixed + Verified + Closed.</t>
         </is>
       </c>
       <c r="C11" s="14" t="n"/>
@@ -1115,7 +1158,7 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Số lỗi lấy toàn bộ từ sheet 05_Lỗi_Tester. "Đang mở" = trạng thái Open + Chưa gửi Dev (chưa xử lý xong).</t>
+          <t>Mục tiêu kỳ do BGD/Tester tự nhập (ô nền vàng), không cố định.</t>
         </is>
       </c>
       <c r="C12" s="14" t="n"/>
@@ -1129,7 +1172,7 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>"Đã xử lý" = Fixed + Verified + Closed. Riêng Deferred (tạm hoãn) tính riêng.</t>
+          <t>Chi tiết theo Trang/Tính năng = mục có Ngày test gần nhất trong kỳ, trạng thái Hoàn thành/Kiểm tra lại.</t>
         </is>
       </c>
       <c r="C13" s="14" t="n"/>
@@ -1143,7 +1186,7 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>Số liệu Database (DN/HR/Ứng viên/Tin TD) lấy từ file Hồ sơ, đếm theo cột ngày.</t>
+          <t>Chỉ số Database lấy từ file Hồ sơ, đếm theo ngày đăng/tạo của kỳ.</t>
         </is>
       </c>
       <c r="C14" s="14" t="n"/>
@@ -1151,40 +1194,41 @@
       <c r="E14" s="14" t="n"/>
       <c r="F14" s="14" t="n"/>
     </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Chỉ số "trong tháng" lọc theo Ngày phát hiện lỗi và Ngày đăng/tạo của kỳ đã chọn.</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>KÍCH HOẠT KẾT NỐI (làm 1 lần)</t>
         </is>
       </c>
-      <c r="B17" s="7" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>① File làm việc QA</t>
+        </is>
+      </c>
+      <c r="B17" s="16">
+        <f>IMPORTRANGE('z_Config'!$B$1,"05_Lỗi_Tester!E4")</f>
+        <v/>
+      </c>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>① File làm việc QA</t>
+          <t>② File Database</t>
         </is>
       </c>
       <c r="B18" s="16">
-        <f>IMPORTRANGE('z_Config'!$B$1,"05_Lỗi_Tester!E4")</f>
+        <f>IMPORTRANGE('z_Config'!$B$3,"'HS DN'!D3")</f>
         <v/>
       </c>
       <c r="C18" s="17" t="n"/>
@@ -1192,69 +1236,70 @@
       <c r="E18" s="17" t="n"/>
       <c r="F18" s="17" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
-        <is>
-          <t>② File Database</t>
-        </is>
-      </c>
-      <c r="B19" s="16">
-        <f>IMPORTRANGE('z_Config'!$B$3,"'HS DN'!D3")</f>
-        <v/>
-      </c>
-      <c r="C19" s="17" t="n"/>
-      <c r="D19" s="17" t="n"/>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-    </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="18" t="inlineStr">
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t>→ Nếu ô ① hoặc ② báo #REF!: bấm vào ô đó → "Cho phép truy cập / Allow access". Làm 1 lần cho mỗi ô.</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n"/>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="5" t="n"/>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="inlineStr">
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Trạng thái kết nối</t>
         </is>
       </c>
-      <c r="B21" s="20">
+      <c r="B20" s="20">
         <f>IF(ISERROR('z_Trang'!$B$1),"⚠ Chưa kết nối file làm việc","✔ Đã kết nối")&amp;"   |   "&amp;IF(ISERROR('z_DB_DN'!$A:$A),"⚠ Chưa kết nối Database","✔ Database OK")</f>
         <v/>
       </c>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>LIÊN KẾT</t>
         </is>
       </c>
-      <c r="B23" s="7" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>File làm việc (QA)</t>
+        </is>
+      </c>
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/spreadsheets/d/1J2A_OiWz7IeYsgafLDY3mIfZsG-xCNGhkNaSQkhicHg/edit</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>File làm việc (QA)</t>
+          <t>File Database (Hồ sơ)</t>
         </is>
       </c>
       <c r="B24" s="21" t="inlineStr">
         <is>
-          <t>https://docs.google.com/spreadsheets/d/1J2A_OiWz7IeYsgafLDY3mIfZsG-xCNGhkNaSQkhicHg/edit</t>
+          <t>https://docs.google.com/spreadsheets/d/1i7-xLYiLHg60EqmCpfeA9B4Y0T-8YsgXk-_0qJ4eACo/edit</t>
         </is>
       </c>
       <c r="C24" s="14" t="n"/>
@@ -1262,73 +1307,53 @@
       <c r="E24" s="14" t="n"/>
       <c r="F24" s="14" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="19" t="inlineStr">
-        <is>
-          <t>File Database (Hồ sơ)</t>
-        </is>
-      </c>
-      <c r="B25" s="21" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/spreadsheets/d/1i7-xLYiLHg60EqmCpfeA9B4Y0T-8YsgXk-_0qJ4eACo/edit</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="25">
-    <mergeCell ref="B25:F25"/>
+  <mergeCells count="24">
+    <mergeCell ref="A16:F16"/>
     <mergeCell ref="C7:F7"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="B21:F21"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="B11:F11"/>
-    <mergeCell ref="A23:F23"/>
     <mergeCell ref="C6:F6"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B14:F14"/>
-    <mergeCell ref="A20:F20"/>
     <mergeCell ref="C5:F5"/>
+    <mergeCell ref="B17:F17"/>
     <mergeCell ref="B13:F13"/>
+    <mergeCell ref="A19:F19"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="B19:F19"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E5A88"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="3" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
   </cols>
@@ -1348,7 +1373,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Chọn tháng ở ô B4. Ô nền vàng là chỉ tiêu nhập tay. Số tổng quan là thời điểm hiện tại; chỉ số "trong tháng" lọc theo tháng đã chọn.</t>
+          <t>Ô nền vàng là mục tiêu nhập tay theo kỳ. Số tổng quan là thời điểm hiện tại; chỉ số "trong tháng" lọc theo kỳ đã chọn.</t>
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
@@ -1400,7 +1425,7 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Mục tiêu tháng</t>
+          <t>Mục tiêu kỳ</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
@@ -1410,7 +1435,7 @@
       </c>
       <c r="D6" s="27" t="inlineStr">
         <is>
-          <t>Tỷ lệ</t>
+          <t>Tỷ lệ đạt</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
@@ -1442,15 +1467,13 @@
           <t>1. Trang hoàn thành</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n">
-        <v>63</v>
-      </c>
+      <c r="B8" s="31" t="n"/>
       <c r="C8" s="32">
         <f>'z_Trang'!$D$1</f>
         <v/>
       </c>
       <c r="D8" s="33">
-        <f>'z_Trang'!$F$1</f>
+        <f>IFERROR(C8/B8,"")</f>
         <v/>
       </c>
       <c r="E8" s="34">
@@ -1459,7 +1482,7 @@
       </c>
       <c r="F8" s="35" t="inlineStr">
         <is>
-          <t>Trên tổng số trang website</t>
+          <t>Hoàn thành / tổng trang</t>
         </is>
       </c>
     </row>
@@ -1469,15 +1492,13 @@
           <t>2. Tính năng hoàn thành</t>
         </is>
       </c>
-      <c r="B9" s="31" t="n">
-        <v>88</v>
-      </c>
+      <c r="B9" s="31" t="n"/>
       <c r="C9" s="37">
         <f>'z_TinhNang'!$D$1</f>
         <v/>
       </c>
       <c r="D9" s="38">
-        <f>'z_TinhNang'!$F$1</f>
+        <f>IFERROR(C9/B9,"")</f>
         <v/>
       </c>
       <c r="E9" s="39">
@@ -1486,7 +1507,7 @@
       </c>
       <c r="F9" s="40" t="inlineStr">
         <is>
-          <t>Trên tổng 88 tính năng</t>
+          <t>Hoàn thành / 88 tính năng</t>
         </is>
       </c>
     </row>
@@ -1496,16 +1517,15 @@
           <t>3. Công việc hoàn thành trong tháng</t>
         </is>
       </c>
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B10" s="31" t="n"/>
       <c r="C10" s="32">
-        <f>COUNTIFS('z_CV'!$B:$B,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_CV'!$B:$B,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_CV'!$O:$O,"Hoàn thành")</f>
-        <v/>
-      </c>
-      <c r="D10" s="41" t="n"/>
+        <f>COUNTIFS('z_CV'!$B:$B,"&gt;="&amp;$N$4,'z_CV'!$B:$B,"&lt;="&amp;$O$4,'z_CV'!$O:$O,"Hoàn thành")</f>
+        <v/>
+      </c>
+      <c r="D10" s="33">
+        <f>IFERROR(C10/B10,"")</f>
+        <v/>
+      </c>
       <c r="E10" s="34">
         <f>IF(ISNUMBER(B10),IF(C10&gt;=B10,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1522,16 +1542,15 @@
           <t>4. Lỗi phát hiện trong tháng</t>
         </is>
       </c>
-      <c r="B11" s="39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B11" s="31" t="n"/>
       <c r="C11" s="37">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4)</f>
-        <v/>
-      </c>
-      <c r="D11" s="42" t="n"/>
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D11" s="38">
+        <f>IFERROR(C11/B11,"")</f>
+        <v/>
+      </c>
       <c r="E11" s="39">
         <f>IF(ISNUMBER(B11),IF(C11&gt;=B11,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1560,16 +1579,15 @@
           <t>1. Lỗi đã xử lý (lũy kế)</t>
         </is>
       </c>
-      <c r="B13" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B13" s="31" t="n"/>
       <c r="C13" s="32">
         <f>(COUNTIF('z_Loi'!$U:$U,"Fixed")+COUNTIF('z_Loi'!$U:$U,"Verified")+COUNTIF('z_Loi'!$U:$U,"Closed"))</f>
         <v/>
       </c>
-      <c r="D13" s="41" t="n"/>
+      <c r="D13" s="33">
+        <f>IFERROR(C13/B13,"")</f>
+        <v/>
+      </c>
       <c r="E13" s="34">
         <f>IF(ISNUMBER(B13),IF(C13&gt;=B13,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1586,16 +1604,15 @@
           <t>2. Số Trang đã xử lý</t>
         </is>
       </c>
-      <c r="B14" s="39" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B14" s="31" t="n"/>
       <c r="C14" s="37">
         <f>'z_Trang'!$B$1-'z_Trang'!$L$1</f>
         <v/>
       </c>
-      <c r="D14" s="42" t="n"/>
+      <c r="D14" s="38">
+        <f>IFERROR(C14/B14,"")</f>
+        <v/>
+      </c>
       <c r="E14" s="39">
         <f>IF(ISNUMBER(B14),IF(C14&gt;=B14,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1612,16 +1629,15 @@
           <t>3. Số Tính năng đã xử lý</t>
         </is>
       </c>
-      <c r="B15" s="34" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="B15" s="31" t="n"/>
       <c r="C15" s="32">
         <f>'z_TinhNang'!$B$1-'z_TinhNang'!$L$1</f>
         <v/>
       </c>
-      <c r="D15" s="41" t="n"/>
+      <c r="D15" s="33">
+        <f>IFERROR(C15/B15,"")</f>
+        <v/>
+      </c>
       <c r="E15" s="34">
         <f>IF(ISNUMBER(B15),IF(C15&gt;=B15,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1650,14 +1666,15 @@
           <t>1. DB Doanh nghiệp đã thêm</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n">
-        <v>100</v>
-      </c>
+      <c r="B17" s="31" t="n"/>
       <c r="C17" s="32">
-        <f>COUNTIFS('z_DB_DN'!$K:$K,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_DB_DN'!$K:$K,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4)</f>
-        <v/>
-      </c>
-      <c r="D17" s="41" t="n"/>
+        <f>COUNTIFS('z_DB_DN'!$K:$K,"&gt;="&amp;$N$4,'z_DB_DN'!$K:$K,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D17" s="33">
+        <f>IFERROR(C17/B17,"")</f>
+        <v/>
+      </c>
       <c r="E17" s="34">
         <f>IF(ISNUMBER(B17),IF(C17&gt;=B17,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1674,14 +1691,15 @@
           <t>2. DB HR đã thêm</t>
         </is>
       </c>
-      <c r="B18" s="31" t="n">
-        <v>100</v>
-      </c>
+      <c r="B18" s="31" t="n"/>
       <c r="C18" s="37">
-        <f>COUNTIFS('z_DB_HR'!$B:$B,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_DB_HR'!$B:$B,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4)</f>
-        <v/>
-      </c>
-      <c r="D18" s="42" t="n"/>
+        <f>COUNTIFS('z_DB_HR'!$B:$B,"&gt;="&amp;$N$4,'z_DB_HR'!$B:$B,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D18" s="38">
+        <f>IFERROR(C18/B18,"")</f>
+        <v/>
+      </c>
       <c r="E18" s="39">
         <f>IF(ISNUMBER(B18),IF(C18&gt;=B18,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1698,14 +1716,15 @@
           <t>3. DB Ứng viên đã thêm</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n">
-        <v>100</v>
-      </c>
+      <c r="B19" s="31" t="n"/>
       <c r="C19" s="32">
         <f>COUNTA('z_DB_UV'!$A:$A)</f>
         <v/>
       </c>
-      <c r="D19" s="41" t="n"/>
+      <c r="D19" s="33">
+        <f>IFERROR(C19/B19,"")</f>
+        <v/>
+      </c>
       <c r="E19" s="34">
         <f>IF(ISNUMBER(B19),IF(C19&gt;=B19,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1722,14 +1741,15 @@
           <t>4. Tin tuyển dụng đã đăng</t>
         </is>
       </c>
-      <c r="B20" s="31" t="n">
-        <v>50</v>
-      </c>
+      <c r="B20" s="31" t="n"/>
       <c r="C20" s="37">
-        <f>COUNTIFS('z_DB_Tin'!$B:$B,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_DB_Tin'!$B:$B,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4)</f>
-        <v/>
-      </c>
-      <c r="D20" s="42" t="n"/>
+        <f>COUNTIFS('z_DB_Tin'!$B:$B,"&gt;="&amp;$N$4,'z_DB_Tin'!$B:$B,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D20" s="38">
+        <f>IFERROR(C20/B20,"")</f>
+        <v/>
+      </c>
       <c r="E20" s="39">
         <f>IF(ISNUMBER(B20),IF(C20&gt;=B20,"Đạt","Chưa đạt"),"Theo dõi")</f>
         <v/>
@@ -1753,22 +1773,22 @@
       <c r="F22" s="7" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="43" t="inlineStr">
+      <c r="A23" s="41" t="inlineStr">
         <is>
           <t>Chỉ số</t>
         </is>
       </c>
-      <c r="B23" s="44" t="inlineStr">
+      <c r="B23" s="42" t="inlineStr">
         <is>
           <t>Số lượng</t>
         </is>
       </c>
-      <c r="C23" s="44" t="inlineStr">
-        <is>
-          <t>Tổng/Mục tiêu</t>
-        </is>
-      </c>
-      <c r="D23" s="44" t="inlineStr">
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
         <is>
           <t>Tỷ lệ</t>
         </is>
@@ -1787,26 +1807,26 @@
       <c r="F24" s="29" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="45" t="inlineStr">
+      <c r="A25" s="43" t="inlineStr">
         <is>
           <t>Trang hoàn thành</t>
         </is>
       </c>
-      <c r="B25" s="46">
+      <c r="B25" s="44">
         <f>'z_Trang'!$D$1</f>
         <v/>
       </c>
-      <c r="C25" s="47">
+      <c r="C25" s="45">
         <f>'z_Trang'!$B$1</f>
         <v/>
       </c>
-      <c r="D25" s="48">
+      <c r="D25" s="46">
         <f>'z_Trang'!$F$1</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="49" t="inlineStr">
+      <c r="A26" s="47" t="inlineStr">
         <is>
           <t>Trang đang kiểm tra</t>
         </is>
@@ -1815,17 +1835,17 @@
         <f>'z_Trang'!$H$1</f>
         <v/>
       </c>
-      <c r="C26" s="50">
+      <c r="C26" s="48">
         <f>'z_Trang'!$B$1</f>
         <v/>
       </c>
-      <c r="D26" s="51">
+      <c r="D26" s="49">
         <f>'z_Trang'!$H$1/'z_Trang'!$B$1</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="52" t="inlineStr">
+      <c r="A27" s="50" t="inlineStr">
         <is>
           <t>Trang cần kiểm tra lại</t>
         </is>
@@ -1834,17 +1854,17 @@
         <f>'z_Trang'!$J$1</f>
         <v/>
       </c>
-      <c r="C27" s="53">
+      <c r="C27" s="51">
         <f>'z_Trang'!$B$1</f>
         <v/>
       </c>
-      <c r="D27" s="54">
+      <c r="D27" s="52">
         <f>'z_Trang'!$J$1/'z_Trang'!$B$1</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="49" t="inlineStr">
+      <c r="A28" s="47" t="inlineStr">
         <is>
           <t>Trang chưa kiểm tra</t>
         </is>
@@ -1853,36 +1873,36 @@
         <f>'z_Trang'!$L$1</f>
         <v/>
       </c>
-      <c r="C28" s="50">
+      <c r="C28" s="48">
         <f>'z_Trang'!$B$1</f>
         <v/>
       </c>
-      <c r="D28" s="51">
+      <c r="D28" s="49">
         <f>'z_Trang'!$L$1/'z_Trang'!$B$1</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="45" t="inlineStr">
+      <c r="A29" s="43" t="inlineStr">
         <is>
           <t>Tính năng hoàn thành</t>
         </is>
       </c>
-      <c r="B29" s="46">
+      <c r="B29" s="44">
         <f>'z_TinhNang'!$D$1</f>
         <v/>
       </c>
-      <c r="C29" s="47">
+      <c r="C29" s="45">
         <f>'z_TinhNang'!$B$1</f>
         <v/>
       </c>
-      <c r="D29" s="48">
+      <c r="D29" s="46">
         <f>'z_TinhNang'!$F$1</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="49" t="inlineStr">
+      <c r="A30" s="47" t="inlineStr">
         <is>
           <t>Tính năng cần kiểm tra lại</t>
         </is>
@@ -1891,17 +1911,17 @@
         <f>'z_TinhNang'!$J$1</f>
         <v/>
       </c>
-      <c r="C30" s="50">
+      <c r="C30" s="48">
         <f>'z_TinhNang'!$B$1</f>
         <v/>
       </c>
-      <c r="D30" s="51">
+      <c r="D30" s="49">
         <f>'z_TinhNang'!$J$1/'z_TinhNang'!$B$1</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="52" t="inlineStr">
+      <c r="A31" s="50" t="inlineStr">
         <is>
           <t>Tính năng chưa kiểm tra</t>
         </is>
@@ -1910,17 +1930,17 @@
         <f>'z_TinhNang'!$L$1</f>
         <v/>
       </c>
-      <c r="C31" s="53">
+      <c r="C31" s="51">
         <f>'z_TinhNang'!$B$1</f>
         <v/>
       </c>
-      <c r="D31" s="54">
+      <c r="D31" s="52">
         <f>'z_TinhNang'!$L$1/'z_TinhNang'!$B$1</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="49" t="inlineStr">
+      <c r="A32" s="47" t="inlineStr">
         <is>
           <t>Tổng lỗi ghi nhận</t>
         </is>
@@ -1929,34 +1949,34 @@
         <f>COUNTA('z_Loi'!$E:$E)-1</f>
         <v/>
       </c>
-      <c r="C32" s="42" t="n"/>
+      <c r="C32" s="53" t="n"/>
       <c r="D32" s="39" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="55" t="inlineStr">
+      <c r="A33" s="54" t="inlineStr">
         <is>
           <t>Lỗi đang mở (Open + Chưa gửi Dev)</t>
         </is>
       </c>
-      <c r="B33" s="56">
+      <c r="B33" s="55">
         <f>(COUNTIF('z_Loi'!$U:$U,"Open")+COUNTIF('z_Loi'!$U:$U,"Chưa gửi Dev"))</f>
         <v/>
       </c>
-      <c r="C33" s="57" t="n"/>
-      <c r="D33" s="58" t="n"/>
+      <c r="C33" s="56" t="n"/>
+      <c r="D33" s="57" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="55" t="inlineStr">
+      <c r="A34" s="54" t="inlineStr">
         <is>
           <t>Lỗi Critical/High đang mở</t>
         </is>
       </c>
-      <c r="B34" s="56">
+      <c r="B34" s="55">
         <f>(COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"High")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"High"))</f>
         <v/>
       </c>
-      <c r="C34" s="57" t="n"/>
-      <c r="D34" s="58" t="n"/>
+      <c r="C34" s="56" t="n"/>
+      <c r="D34" s="57" t="n"/>
     </row>
     <row r="35" ht="19" customHeight="1">
       <c r="A35" s="28" t="inlineStr">
@@ -1971,7 +1991,7 @@
       <c r="F35" s="29" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="52" t="inlineStr">
+      <c r="A36" s="50" t="inlineStr">
         <is>
           <t>DB Doanh nghiệp</t>
         </is>
@@ -1980,11 +2000,11 @@
         <f>COUNTA('z_DB_DN'!$A:$A)</f>
         <v/>
       </c>
-      <c r="C36" s="41" t="n"/>
+      <c r="C36" s="58" t="n"/>
       <c r="D36" s="34" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="49" t="inlineStr">
+      <c r="A37" s="47" t="inlineStr">
         <is>
           <t>DB HR</t>
         </is>
@@ -1993,11 +2013,11 @@
         <f>COUNTA('z_DB_HR'!$A:$A)</f>
         <v/>
       </c>
-      <c r="C37" s="42" t="n"/>
+      <c r="C37" s="53" t="n"/>
       <c r="D37" s="39" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="52" t="inlineStr">
+      <c r="A38" s="50" t="inlineStr">
         <is>
           <t>DB Ứng viên</t>
         </is>
@@ -2006,11 +2026,11 @@
         <f>COUNTA('z_DB_UV'!$A:$A)</f>
         <v/>
       </c>
-      <c r="C38" s="41" t="n"/>
+      <c r="C38" s="58" t="n"/>
       <c r="D38" s="34" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="49" t="inlineStr">
+      <c r="A39" s="47" t="inlineStr">
         <is>
           <t>Tin tuyển dụng đã đăng</t>
         </is>
@@ -2019,7 +2039,7 @@
         <f>COUNTA('z_DB_Tin'!$A:$A)</f>
         <v/>
       </c>
-      <c r="C39" s="42" t="n"/>
+      <c r="C39" s="53" t="n"/>
       <c r="D39" s="39" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
@@ -2035,17 +2055,17 @@
       <c r="F41" s="7" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="43" t="inlineStr">
+      <c r="A42" s="41" t="inlineStr">
         <is>
           <t>Trạng thái</t>
         </is>
       </c>
-      <c r="B42" s="44" t="inlineStr">
+      <c r="B42" s="42" t="inlineStr">
         <is>
           <t>Số lỗi</t>
         </is>
       </c>
-      <c r="C42" s="43" t="inlineStr">
+      <c r="C42" s="41" t="inlineStr">
         <is>
           <t>Ý nghĩa</t>
         </is>
@@ -2171,7 +2191,7 @@
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>PHÂN BỐ LỖI TRONG THÁNG</t>
+          <t>PHÂN BỐ LỖI PHÁT HIỆN TRONG THÁNG</t>
         </is>
       </c>
       <c r="B50" s="7" t="n"/>
@@ -2181,22 +2201,22 @@
       <c r="F50" s="7" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="43" t="inlineStr">
+      <c r="A51" s="41" t="inlineStr">
         <is>
           <t>Theo mức độ</t>
         </is>
       </c>
-      <c r="B51" s="44" t="inlineStr">
+      <c r="B51" s="42" t="inlineStr">
         <is>
           <t>Số lỗi</t>
         </is>
       </c>
-      <c r="D51" s="43" t="inlineStr">
+      <c r="D51" s="41" t="inlineStr">
         <is>
           <t>Theo thiết bị</t>
         </is>
       </c>
-      <c r="E51" s="44" t="inlineStr">
+      <c r="E51" s="42" t="inlineStr">
         <is>
           <t>Số lỗi</t>
         </is>
@@ -2209,16 +2229,16 @@
         </is>
       </c>
       <c r="B52" s="32">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$L:$L,"Critical")</f>
-        <v/>
-      </c>
-      <c r="D52" s="52" t="inlineStr">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Critical")</f>
+        <v/>
+      </c>
+      <c r="D52" s="50" t="inlineStr">
         <is>
           <t>Desktop</t>
         </is>
       </c>
       <c r="E52" s="32">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$M:$M,"*Desktop*")</f>
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Desktop*")</f>
         <v/>
       </c>
     </row>
@@ -2229,16 +2249,16 @@
         </is>
       </c>
       <c r="B53" s="37">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$L:$L,"High")</f>
-        <v/>
-      </c>
-      <c r="D53" s="49" t="inlineStr">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"High")</f>
+        <v/>
+      </c>
+      <c r="D53" s="47" t="inlineStr">
         <is>
           <t>Mobile</t>
         </is>
       </c>
       <c r="E53" s="37">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$M:$M,"*Mobile*")</f>
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Mobile*")</f>
         <v/>
       </c>
     </row>
@@ -2249,16 +2269,16 @@
         </is>
       </c>
       <c r="B54" s="32">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$L:$L,"Medium")</f>
-        <v/>
-      </c>
-      <c r="D54" s="52" t="inlineStr">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Medium")</f>
+        <v/>
+      </c>
+      <c r="D54" s="50" t="inlineStr">
         <is>
           <t>Tablet</t>
         </is>
       </c>
       <c r="E54" s="32">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$M:$M,"*Tablet*")</f>
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Tablet*")</f>
         <v/>
       </c>
     </row>
@@ -2269,7 +2289,7 @@
         </is>
       </c>
       <c r="B55" s="37">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;'01_Báo_cáo_Tháng'!$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;'01_Báo_cáo_Tháng'!$O$4,'z_Loi'!$L:$L,"Low")</f>
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Low")</f>
         <v/>
       </c>
     </row>
@@ -2318,7 +2338,7 @@
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="11" t="inlineStr">
         <is>
-          <t>CHI TIẾT LỖI TRONG THÁNG THEO TRANG &amp; TÍNH NĂNG</t>
+          <t>CHI TIẾT: TRANG &amp; TÍNH NĂNG ĐÃ TEST TRONG THÁNG</t>
         </is>
       </c>
       <c r="B61" s="7" t="n"/>
@@ -2328,125 +2348,829 @@
       <c r="F61" s="7" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="43" t="inlineStr">
-        <is>
-          <t>Trang đã kiểm thử trong tháng</t>
-        </is>
-      </c>
-      <c r="B62" s="44" t="inlineStr">
+      <c r="A62" s="77" t="inlineStr">
+        <is>
+          <t>Liệt kê các trang/tính năng có Ngày test gần nhất trong kỳ (trạng thái Hoàn thành hoặc Kiểm tra lại).</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="n"/>
+      <c r="C62" s="5" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
+      <c r="F62" s="5" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="41" t="inlineStr">
+        <is>
+          <t>TRANG đã test trong kỳ</t>
+        </is>
+      </c>
+      <c r="B63" s="42" t="inlineStr">
         <is>
           <t>Số lỗi</t>
         </is>
       </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Tính năng đã kiểm thử trong tháng</t>
-        </is>
-      </c>
-      <c r="E62" s="44" t="inlineStr">
-        <is>
-          <t>Số lỗi</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="77">
-        <f>IFERROR(QUERY('z_Loi'!$A$1:$U$606,"select B, count(E) where E is not null and Q &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and Q &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' group by B order by count(E) desc label count(E) '', B ''",1),"(không có lỗi trong kỳ)")</f>
-        <v/>
-      </c>
-      <c r="B63" s="14" t="n"/>
-      <c r="D63" s="77">
-        <f>IFERROR(QUERY('z_Loi'!$A$1:$U$606,"select D, count(E) where E is not null and Q &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and Q &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' group by D order by count(E) desc label count(E) '', D ''",1),"(không có lỗi trong kỳ)")</f>
-        <v/>
-      </c>
-      <c r="E63" s="14" t="n"/>
+      <c r="C63" s="42" t="inlineStr">
+        <is>
+          <t>Ngày test/retest</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="n"/>
-      <c r="B64" s="14" t="n"/>
-      <c r="D64" s="14" t="n"/>
-      <c r="E64" s="14" t="n"/>
+      <c r="A64" s="78">
+        <f>IFERROR(QUERY('z_TrangFull'!$A$1:$R$65,"select B, I, P where P &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and P &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' and (E = 'Hoàn thành' or E = 'Kiểm tra lại') order by P desc label B '', I '', P '' format P 'dd/mm/yyyy', I '#,##0'",1),"(không có trang test trong kỳ)")</f>
+        <v/>
+      </c>
+      <c r="B64" s="79" t="n"/>
+      <c r="C64" s="80" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="14" t="n"/>
-      <c r="B65" s="14" t="n"/>
-      <c r="D65" s="14" t="n"/>
-      <c r="E65" s="14" t="n"/>
+      <c r="B65" s="79" t="n"/>
+      <c r="C65" s="80" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="14" t="n"/>
-      <c r="B66" s="14" t="n"/>
-      <c r="D66" s="14" t="n"/>
-      <c r="E66" s="14" t="n"/>
+      <c r="B66" s="79" t="n"/>
+      <c r="C66" s="80" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="14" t="n"/>
-      <c r="B67" s="14" t="n"/>
-      <c r="D67" s="14" t="n"/>
-      <c r="E67" s="14" t="n"/>
+      <c r="B67" s="79" t="n"/>
+      <c r="C67" s="80" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="14" t="n"/>
-      <c r="B68" s="14" t="n"/>
-      <c r="D68" s="14" t="n"/>
-      <c r="E68" s="14" t="n"/>
+      <c r="B68" s="79" t="n"/>
+      <c r="C68" s="80" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="14" t="n"/>
-      <c r="B69" s="14" t="n"/>
-      <c r="D69" s="14" t="n"/>
-      <c r="E69" s="14" t="n"/>
+      <c r="B69" s="79" t="n"/>
+      <c r="C69" s="80" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="14" t="n"/>
-      <c r="B70" s="14" t="n"/>
-      <c r="D70" s="14" t="n"/>
-      <c r="E70" s="14" t="n"/>
+      <c r="B70" s="79" t="n"/>
+      <c r="C70" s="80" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="14" t="n"/>
-      <c r="B71" s="14" t="n"/>
-      <c r="D71" s="14" t="n"/>
-      <c r="E71" s="14" t="n"/>
+      <c r="B71" s="79" t="n"/>
+      <c r="C71" s="80" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="14" t="n"/>
-      <c r="B72" s="14" t="n"/>
-      <c r="D72" s="14" t="n"/>
-      <c r="E72" s="14" t="n"/>
+      <c r="B72" s="79" t="n"/>
+      <c r="C72" s="80" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="14" t="n"/>
-      <c r="B73" s="14" t="n"/>
-      <c r="D73" s="14" t="n"/>
-      <c r="E73" s="14" t="n"/>
+      <c r="B73" s="79" t="n"/>
+      <c r="C73" s="80" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="14" t="n"/>
-      <c r="B74" s="14" t="n"/>
-      <c r="D74" s="14" t="n"/>
-      <c r="E74" s="14" t="n"/>
+      <c r="B74" s="79" t="n"/>
+      <c r="C74" s="80" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="14" t="n"/>
-      <c r="B75" s="14" t="n"/>
-      <c r="D75" s="14" t="n"/>
-      <c r="E75" s="14" t="n"/>
+      <c r="B75" s="79" t="n"/>
+      <c r="C75" s="80" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="14" t="n"/>
-      <c r="B76" s="14" t="n"/>
-      <c r="D76" s="14" t="n"/>
-      <c r="E76" s="14" t="n"/>
+      <c r="B76" s="79" t="n"/>
+      <c r="C76" s="80" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="14" t="n"/>
-      <c r="B77" s="14" t="n"/>
-      <c r="D77" s="14" t="n"/>
-      <c r="E77" s="14" t="n"/>
+      <c r="B77" s="79" t="n"/>
+      <c r="C77" s="80" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="n"/>
+      <c r="B78" s="79" t="n"/>
+      <c r="C78" s="80" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="n"/>
+      <c r="B79" s="79" t="n"/>
+      <c r="C79" s="80" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="n"/>
+      <c r="B80" s="79" t="n"/>
+      <c r="C80" s="80" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n"/>
+      <c r="B81" s="79" t="n"/>
+      <c r="C81" s="80" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="n"/>
+      <c r="B82" s="79" t="n"/>
+      <c r="C82" s="80" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="n"/>
+      <c r="B83" s="79" t="n"/>
+      <c r="C83" s="80" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="n"/>
+      <c r="B84" s="79" t="n"/>
+      <c r="C84" s="80" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="n"/>
+      <c r="B85" s="79" t="n"/>
+      <c r="C85" s="80" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="n"/>
+      <c r="B86" s="79" t="n"/>
+      <c r="C86" s="80" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="n"/>
+      <c r="B87" s="79" t="n"/>
+      <c r="C87" s="80" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="n"/>
+      <c r="B88" s="79" t="n"/>
+      <c r="C88" s="80" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="n"/>
+      <c r="B89" s="79" t="n"/>
+      <c r="C89" s="80" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="n"/>
+      <c r="B90" s="79" t="n"/>
+      <c r="C90" s="80" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="n"/>
+      <c r="B91" s="79" t="n"/>
+      <c r="C91" s="80" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="n"/>
+      <c r="B92" s="79" t="n"/>
+      <c r="C92" s="80" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="n"/>
+      <c r="B93" s="79" t="n"/>
+      <c r="C93" s="80" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="n"/>
+      <c r="B94" s="79" t="n"/>
+      <c r="C94" s="80" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="n"/>
+      <c r="B95" s="79" t="n"/>
+      <c r="C95" s="80" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="n"/>
+      <c r="B96" s="79" t="n"/>
+      <c r="C96" s="80" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="n"/>
+      <c r="B97" s="79" t="n"/>
+      <c r="C97" s="80" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="n"/>
+      <c r="B98" s="79" t="n"/>
+      <c r="C98" s="80" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="n"/>
+      <c r="B99" s="79" t="n"/>
+      <c r="C99" s="80" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="n"/>
+      <c r="B100" s="79" t="n"/>
+      <c r="C100" s="80" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="n"/>
+      <c r="B101" s="79" t="n"/>
+      <c r="C101" s="80" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="n"/>
+      <c r="B102" s="79" t="n"/>
+      <c r="C102" s="80" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="n"/>
+      <c r="B103" s="79" t="n"/>
+      <c r="C103" s="80" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="n"/>
+      <c r="B104" s="79" t="n"/>
+      <c r="C104" s="80" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="n"/>
+      <c r="B105" s="79" t="n"/>
+      <c r="C105" s="80" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="n"/>
+      <c r="B106" s="79" t="n"/>
+      <c r="C106" s="80" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="n"/>
+      <c r="B107" s="79" t="n"/>
+      <c r="C107" s="80" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="n"/>
+      <c r="B108" s="79" t="n"/>
+      <c r="C108" s="80" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="n"/>
+      <c r="B109" s="79" t="n"/>
+      <c r="C109" s="80" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="n"/>
+      <c r="B110" s="79" t="n"/>
+      <c r="C110" s="80" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="n"/>
+      <c r="B111" s="79" t="n"/>
+      <c r="C111" s="80" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="n"/>
+      <c r="B112" s="79" t="n"/>
+      <c r="C112" s="80" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="n"/>
+      <c r="B113" s="79" t="n"/>
+      <c r="C113" s="80" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="n"/>
+      <c r="B114" s="79" t="n"/>
+      <c r="C114" s="80" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="n"/>
+      <c r="B115" s="79" t="n"/>
+      <c r="C115" s="80" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="n"/>
+      <c r="B116" s="79" t="n"/>
+      <c r="C116" s="80" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="14" t="n"/>
+      <c r="B117" s="79" t="n"/>
+      <c r="C117" s="80" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="n"/>
+      <c r="B118" s="79" t="n"/>
+      <c r="C118" s="80" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="n"/>
+      <c r="B119" s="79" t="n"/>
+      <c r="C119" s="80" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="n"/>
+      <c r="B120" s="79" t="n"/>
+      <c r="C120" s="80" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="n"/>
+      <c r="B121" s="79" t="n"/>
+      <c r="C121" s="80" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="n"/>
+      <c r="B122" s="79" t="n"/>
+      <c r="C122" s="80" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="14" t="n"/>
+      <c r="B123" s="79" t="n"/>
+      <c r="C123" s="80" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="n"/>
+      <c r="B124" s="79" t="n"/>
+      <c r="C124" s="80" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="n"/>
+      <c r="B125" s="79" t="n"/>
+      <c r="C125" s="80" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="n"/>
+      <c r="B126" s="79" t="n"/>
+      <c r="C126" s="80" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="n"/>
+      <c r="B127" s="79" t="n"/>
+      <c r="C127" s="80" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="41" t="inlineStr">
+        <is>
+          <t>TÍNH NĂNG đã test trong kỳ</t>
+        </is>
+      </c>
+      <c r="B129" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+      <c r="C129" s="42" t="inlineStr">
+        <is>
+          <t>Ngày test/retest</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="78">
+        <f>IFERROR(QUERY('z_TNFull'!$A$1:$T$89,"select B, K, R where R &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and R &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' and (J = 'Hoàn thành' or J = 'Kiểm tra lại') order by R desc label B '', K '', R '' format R 'dd/mm/yyyy', K '#,##0'",1),"(không có tính năng test trong kỳ)")</f>
+        <v/>
+      </c>
+      <c r="B130" s="79" t="n"/>
+      <c r="C130" s="80" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="14" t="n"/>
+      <c r="B131" s="79" t="n"/>
+      <c r="C131" s="80" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="n"/>
+      <c r="B132" s="79" t="n"/>
+      <c r="C132" s="80" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="n"/>
+      <c r="B133" s="79" t="n"/>
+      <c r="C133" s="80" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="n"/>
+      <c r="B134" s="79" t="n"/>
+      <c r="C134" s="80" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="n"/>
+      <c r="B135" s="79" t="n"/>
+      <c r="C135" s="80" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="n"/>
+      <c r="B136" s="79" t="n"/>
+      <c r="C136" s="80" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="n"/>
+      <c r="B137" s="79" t="n"/>
+      <c r="C137" s="80" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="n"/>
+      <c r="B138" s="79" t="n"/>
+      <c r="C138" s="80" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="n"/>
+      <c r="B139" s="79" t="n"/>
+      <c r="C139" s="80" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="n"/>
+      <c r="B140" s="79" t="n"/>
+      <c r="C140" s="80" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="n"/>
+      <c r="B141" s="79" t="n"/>
+      <c r="C141" s="80" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="n"/>
+      <c r="B142" s="79" t="n"/>
+      <c r="C142" s="80" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="14" t="n"/>
+      <c r="B143" s="79" t="n"/>
+      <c r="C143" s="80" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="14" t="n"/>
+      <c r="B144" s="79" t="n"/>
+      <c r="C144" s="80" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="14" t="n"/>
+      <c r="B145" s="79" t="n"/>
+      <c r="C145" s="80" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="n"/>
+      <c r="B146" s="79" t="n"/>
+      <c r="C146" s="80" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="14" t="n"/>
+      <c r="B147" s="79" t="n"/>
+      <c r="C147" s="80" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="n"/>
+      <c r="B148" s="79" t="n"/>
+      <c r="C148" s="80" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="n"/>
+      <c r="B149" s="79" t="n"/>
+      <c r="C149" s="80" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="n"/>
+      <c r="B150" s="79" t="n"/>
+      <c r="C150" s="80" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="n"/>
+      <c r="B151" s="79" t="n"/>
+      <c r="C151" s="80" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="14" t="n"/>
+      <c r="B152" s="79" t="n"/>
+      <c r="C152" s="80" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="14" t="n"/>
+      <c r="B153" s="79" t="n"/>
+      <c r="C153" s="80" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="14" t="n"/>
+      <c r="B154" s="79" t="n"/>
+      <c r="C154" s="80" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="14" t="n"/>
+      <c r="B155" s="79" t="n"/>
+      <c r="C155" s="80" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="14" t="n"/>
+      <c r="B156" s="79" t="n"/>
+      <c r="C156" s="80" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="14" t="n"/>
+      <c r="B157" s="79" t="n"/>
+      <c r="C157" s="80" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="14" t="n"/>
+      <c r="B158" s="79" t="n"/>
+      <c r="C158" s="80" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="14" t="n"/>
+      <c r="B159" s="79" t="n"/>
+      <c r="C159" s="80" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="14" t="n"/>
+      <c r="B160" s="79" t="n"/>
+      <c r="C160" s="80" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="14" t="n"/>
+      <c r="B161" s="79" t="n"/>
+      <c r="C161" s="80" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="14" t="n"/>
+      <c r="B162" s="79" t="n"/>
+      <c r="C162" s="80" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="14" t="n"/>
+      <c r="B163" s="79" t="n"/>
+      <c r="C163" s="80" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="14" t="n"/>
+      <c r="B164" s="79" t="n"/>
+      <c r="C164" s="80" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="14" t="n"/>
+      <c r="B165" s="79" t="n"/>
+      <c r="C165" s="80" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="14" t="n"/>
+      <c r="B166" s="79" t="n"/>
+      <c r="C166" s="80" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="14" t="n"/>
+      <c r="B167" s="79" t="n"/>
+      <c r="C167" s="80" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="14" t="n"/>
+      <c r="B168" s="79" t="n"/>
+      <c r="C168" s="80" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="14" t="n"/>
+      <c r="B169" s="79" t="n"/>
+      <c r="C169" s="80" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="14" t="n"/>
+      <c r="B170" s="79" t="n"/>
+      <c r="C170" s="80" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="14" t="n"/>
+      <c r="B171" s="79" t="n"/>
+      <c r="C171" s="80" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="14" t="n"/>
+      <c r="B172" s="79" t="n"/>
+      <c r="C172" s="80" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="14" t="n"/>
+      <c r="B173" s="79" t="n"/>
+      <c r="C173" s="80" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="14" t="n"/>
+      <c r="B174" s="79" t="n"/>
+      <c r="C174" s="80" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="14" t="n"/>
+      <c r="B175" s="79" t="n"/>
+      <c r="C175" s="80" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="14" t="n"/>
+      <c r="B176" s="79" t="n"/>
+      <c r="C176" s="80" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="14" t="n"/>
+      <c r="B177" s="79" t="n"/>
+      <c r="C177" s="80" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="14" t="n"/>
+      <c r="B178" s="79" t="n"/>
+      <c r="C178" s="80" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="14" t="n"/>
+      <c r="B179" s="79" t="n"/>
+      <c r="C179" s="80" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="14" t="n"/>
+      <c r="B180" s="79" t="n"/>
+      <c r="C180" s="80" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="14" t="n"/>
+      <c r="B181" s="79" t="n"/>
+      <c r="C181" s="80" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="14" t="n"/>
+      <c r="B182" s="79" t="n"/>
+      <c r="C182" s="80" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="14" t="n"/>
+      <c r="B183" s="79" t="n"/>
+      <c r="C183" s="80" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="14" t="n"/>
+      <c r="B184" s="79" t="n"/>
+      <c r="C184" s="80" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="14" t="n"/>
+      <c r="B185" s="79" t="n"/>
+      <c r="C185" s="80" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="14" t="n"/>
+      <c r="B186" s="79" t="n"/>
+      <c r="C186" s="80" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="14" t="n"/>
+      <c r="B187" s="79" t="n"/>
+      <c r="C187" s="80" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="14" t="n"/>
+      <c r="B188" s="79" t="n"/>
+      <c r="C188" s="80" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="14" t="n"/>
+      <c r="B189" s="79" t="n"/>
+      <c r="C189" s="80" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="14" t="n"/>
+      <c r="B190" s="79" t="n"/>
+      <c r="C190" s="80" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="14" t="n"/>
+      <c r="B191" s="79" t="n"/>
+      <c r="C191" s="80" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="14" t="n"/>
+      <c r="B192" s="79" t="n"/>
+      <c r="C192" s="80" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="14" t="n"/>
+      <c r="B193" s="79" t="n"/>
+      <c r="C193" s="80" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="14" t="n"/>
+      <c r="B194" s="79" t="n"/>
+      <c r="C194" s="80" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="14" t="n"/>
+      <c r="B195" s="79" t="n"/>
+      <c r="C195" s="80" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="14" t="n"/>
+      <c r="B196" s="79" t="n"/>
+      <c r="C196" s="80" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="14" t="n"/>
+      <c r="B197" s="79" t="n"/>
+      <c r="C197" s="80" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="14" t="n"/>
+      <c r="B198" s="79" t="n"/>
+      <c r="C198" s="80" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="14" t="n"/>
+      <c r="B199" s="79" t="n"/>
+      <c r="C199" s="80" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="14" t="n"/>
+      <c r="B200" s="79" t="n"/>
+      <c r="C200" s="80" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="14" t="n"/>
+      <c r="B201" s="79" t="n"/>
+      <c r="C201" s="80" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="14" t="n"/>
+      <c r="B202" s="79" t="n"/>
+      <c r="C202" s="80" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="14" t="n"/>
+      <c r="B203" s="79" t="n"/>
+      <c r="C203" s="80" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="14" t="n"/>
+      <c r="B204" s="79" t="n"/>
+      <c r="C204" s="80" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="14" t="n"/>
+      <c r="B205" s="79" t="n"/>
+      <c r="C205" s="80" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="14" t="n"/>
+      <c r="B206" s="79" t="n"/>
+      <c r="C206" s="80" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="14" t="n"/>
+      <c r="B207" s="79" t="n"/>
+      <c r="C207" s="80" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="n"/>
+      <c r="B208" s="79" t="n"/>
+      <c r="C208" s="80" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="14" t="n"/>
+      <c r="B209" s="79" t="n"/>
+      <c r="C209" s="80" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="14" t="n"/>
+      <c r="B210" s="79" t="n"/>
+      <c r="C210" s="80" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="14" t="n"/>
+      <c r="B211" s="79" t="n"/>
+      <c r="C211" s="80" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="14" t="n"/>
+      <c r="B212" s="79" t="n"/>
+      <c r="C212" s="80" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="14" t="n"/>
+      <c r="B213" s="79" t="n"/>
+      <c r="C213" s="80" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="14" t="n"/>
+      <c r="B214" s="79" t="n"/>
+      <c r="C214" s="80" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="14" t="n"/>
+      <c r="B215" s="79" t="n"/>
+      <c r="C215" s="80" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="14" t="n"/>
+      <c r="B216" s="79" t="n"/>
+      <c r="C216" s="80" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="14" t="n"/>
+      <c r="B217" s="79" t="n"/>
+      <c r="C217" s="80" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="14" t="n"/>
+      <c r="B218" s="79" t="n"/>
+      <c r="C218" s="80" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="14" t="n"/>
+      <c r="B219" s="79" t="n"/>
+      <c r="C219" s="80" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
+  <mergeCells count="22">
     <mergeCell ref="A41:F41"/>
     <mergeCell ref="A16:F16"/>
     <mergeCell ref="C48:F48"/>
@@ -2458,6 +3182,7 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A62:F62"/>
     <mergeCell ref="C42:F42"/>
     <mergeCell ref="C45:F45"/>
     <mergeCell ref="C47:F47"/>
@@ -2478,22 +3203,22 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002E7D32"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
+  <dimension ref="A1:O220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col hidden="1" width="13" customWidth="1" min="14" max="14"/>
     <col hidden="1" width="13" customWidth="1" min="15" max="15"/>
   </cols>
@@ -2513,7 +3238,7 @@
     <row r="2">
       <c r="A2" s="22" t="inlineStr">
         <is>
-          <t>Tuần theo tuần-trong-tháng: Tuần 1 = ngày 1–7, Tuần 2 = 8–14, ...</t>
+          <t>Ô nền vàng là mục tiêu nhập tay theo kỳ. Số tổng quan là thời điểm hiện tại; chỉ số "trong tuần" lọc theo kỳ đã chọn.</t>
         </is>
       </c>
       <c r="B2" s="5" t="n"/>
@@ -2557,319 +3282,1807 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="inlineStr">
+      <c r="A5" s="81" t="inlineStr">
         <is>
           <t>Từ ngày</t>
         </is>
       </c>
-      <c r="B5" s="79">
+      <c r="B5" s="82">
         <f>N4</f>
         <v/>
       </c>
-      <c r="C5" s="78" t="inlineStr">
+      <c r="C5" s="81" t="inlineStr">
         <is>
           <t>Đến ngày</t>
         </is>
       </c>
-      <c r="D5" s="79">
+      <c r="D5" s="83">
         <f>O4</f>
         <v/>
       </c>
-      <c r="E5" s="80">
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="84">
         <f>IF(ISERROR('z_Trang'!$B$1),"⚠ Chưa kết nối","✔ Đã kết nối")</f>
         <v/>
       </c>
-      <c r="F5" s="5" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>CHỈ SỐ TRONG TUẦN</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>KPI / CHỈ SỐ</t>
+        </is>
+      </c>
+      <c r="B7" s="27" t="inlineStr">
+        <is>
+          <t>Mục tiêu kỳ</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Kết quả</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Tỷ lệ đạt</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Đạt KPI?</t>
+        </is>
+      </c>
+      <c r="F7" s="27" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="28" t="inlineStr">
+        <is>
+          <t>I. KIỂM TRA WEBSITE</t>
+        </is>
+      </c>
+      <c r="B8" s="29" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="29" t="n"/>
+      <c r="F8" s="29" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="30" t="inlineStr">
+        <is>
+          <t>1. Trang hoàn thành</t>
+        </is>
+      </c>
+      <c r="B9" s="31" t="n"/>
+      <c r="C9" s="32">
+        <f>'z_Trang'!$D$1</f>
+        <v/>
+      </c>
+      <c r="D9" s="33">
+        <f>IFERROR(C9/B9,"")</f>
+        <v/>
+      </c>
+      <c r="E9" s="34">
+        <f>IF(ISNUMBER(B9),IF(C9&gt;=B9,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F9" s="35" t="inlineStr">
+        <is>
+          <t>Hoàn thành / tổng trang</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="36" t="inlineStr">
+        <is>
+          <t>2. Tính năng hoàn thành</t>
+        </is>
+      </c>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="37">
+        <f>'z_TinhNang'!$D$1</f>
+        <v/>
+      </c>
+      <c r="D10" s="38">
+        <f>IFERROR(C10/B10,"")</f>
+        <v/>
+      </c>
+      <c r="E10" s="39">
+        <f>IF(ISNUMBER(B10),IF(C10&gt;=B10,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F10" s="40" t="inlineStr">
+        <is>
+          <t>Hoàn thành / 88 tính năng</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="30" t="inlineStr">
+        <is>
+          <t>3. Công việc hoàn thành trong tuần</t>
+        </is>
+      </c>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="32">
+        <f>COUNTIFS('z_CV'!$B:$B,"&gt;="&amp;$N$4,'z_CV'!$B:$B,"&lt;="&amp;$O$4,'z_CV'!$O:$O,"Hoàn thành")</f>
+        <v/>
+      </c>
+      <c r="D11" s="33">
+        <f>IFERROR(C11/B11,"")</f>
+        <v/>
+      </c>
+      <c r="E11" s="34">
+        <f>IF(ISNUMBER(B11),IF(C11&gt;=B11,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F11" s="35" t="inlineStr">
+        <is>
+          <t>Nhật ký công việc theo ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="36" t="inlineStr">
+        <is>
+          <t>4. Lỗi phát hiện trong tuần</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="37">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D12" s="38">
+        <f>IFERROR(C12/B12,"")</f>
+        <v/>
+      </c>
+      <c r="E12" s="39">
+        <f>IF(ISNUMBER(B12),IF(C12&gt;=B12,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F12" s="40" t="inlineStr">
+        <is>
+          <t>Theo Ngày phát hiện (05_Lỗi_Tester)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="19" customHeight="1">
+      <c r="A13" s="28" t="inlineStr">
+        <is>
+          <t>II. HOÀN THIỆN WEBSITE</t>
+        </is>
+      </c>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="30" t="inlineStr">
+        <is>
+          <t>1. Lỗi đã xử lý (lũy kế)</t>
+        </is>
+      </c>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="32">
+        <f>(COUNTIF('z_Loi'!$U:$U,"Fixed")+COUNTIF('z_Loi'!$U:$U,"Verified")+COUNTIF('z_Loi'!$U:$U,"Closed"))</f>
+        <v/>
+      </c>
+      <c r="D14" s="33">
+        <f>IFERROR(C14/B14,"")</f>
+        <v/>
+      </c>
+      <c r="E14" s="34">
+        <f>IF(ISNUMBER(B14),IF(C14&gt;=B14,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F14" s="35" t="inlineStr">
+        <is>
+          <t>Fixed + Verified + Closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="36" t="inlineStr">
+        <is>
+          <t>2. Số Trang đã xử lý</t>
+        </is>
+      </c>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="37">
+        <f>'z_Trang'!$B$1-'z_Trang'!$L$1</f>
+        <v/>
+      </c>
+      <c r="D15" s="38">
+        <f>IFERROR(C15/B15,"")</f>
+        <v/>
+      </c>
+      <c r="E15" s="39">
+        <f>IF(ISNUMBER(B15),IF(C15&gt;=B15,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F15" s="40" t="inlineStr">
+        <is>
+          <t>Đã kiểm thử = Tổng − Chưa kiểm tra</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="30" t="inlineStr">
+        <is>
+          <t>3. Số Tính năng đã xử lý</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="32">
+        <f>'z_TinhNang'!$B$1-'z_TinhNang'!$L$1</f>
+        <v/>
+      </c>
+      <c r="D16" s="33">
+        <f>IFERROR(C16/B16,"")</f>
+        <v/>
+      </c>
+      <c r="E16" s="34">
+        <f>IF(ISNUMBER(B16),IF(C16&gt;=B16,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F16" s="35" t="inlineStr">
+        <is>
+          <t>Đã kiểm thử = Tổng − Chưa kiểm tra</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="19" customHeight="1">
+      <c r="A17" s="28" t="inlineStr">
+        <is>
+          <t>III. DATABASE (trong tuần)</t>
+        </is>
+      </c>
+      <c r="B17" s="29" t="n"/>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="29" t="n"/>
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="30" t="inlineStr">
+        <is>
+          <t>1. DB Doanh nghiệp đã thêm</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="32">
+        <f>COUNTIFS('z_DB_DN'!$K:$K,"&gt;="&amp;$N$4,'z_DB_DN'!$K:$K,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D18" s="33">
+        <f>IFERROR(C18/B18,"")</f>
+        <v/>
+      </c>
+      <c r="E18" s="34">
+        <f>IF(ISNUMBER(B18),IF(C18&gt;=B18,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F18" s="35" t="inlineStr">
+        <is>
+          <t>Theo Ngày Đăng/Tạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="36" t="inlineStr">
+        <is>
+          <t>2. DB HR đã thêm</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="37">
+        <f>COUNTIFS('z_DB_HR'!$B:$B,"&gt;="&amp;$N$4,'z_DB_HR'!$B:$B,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D19" s="38">
+        <f>IFERROR(C19/B19,"")</f>
+        <v/>
+      </c>
+      <c r="E19" s="39">
+        <f>IF(ISNUMBER(B19),IF(C19&gt;=B19,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F19" s="40" t="inlineStr">
+        <is>
+          <t>Theo Ngày Đăng/Tạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="30" t="inlineStr">
+        <is>
+          <t>3. DB Ứng viên đã thêm</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="32">
+        <f>COUNTA('z_DB_UV'!$A:$A)</f>
+        <v/>
+      </c>
+      <c r="D20" s="33">
+        <f>IFERROR(C20/B20,"")</f>
+        <v/>
+      </c>
+      <c r="E20" s="34">
+        <f>IF(ISNUMBER(B20),IF(C20&gt;=B20,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>Theo tổng (chưa có cột ngày nhập)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="36" t="inlineStr">
+        <is>
+          <t>4. Tin tuyển dụng đã đăng</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="37">
+        <f>COUNTIFS('z_DB_Tin'!$B:$B,"&gt;="&amp;$N$4,'z_DB_Tin'!$B:$B,"&lt;="&amp;$O$4)</f>
+        <v/>
+      </c>
+      <c r="D21" s="38">
+        <f>IFERROR(C21/B21,"")</f>
+        <v/>
+      </c>
+      <c r="E21" s="39">
+        <f>IF(ISNUMBER(B21),IF(C21&gt;=B21,"Đạt","Chưa đạt"),"Theo dõi")</f>
+        <v/>
+      </c>
+      <c r="F21" s="40" t="inlineStr">
+        <is>
+          <t>Theo Ngày viết</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>TỔNG QUAN HIỆN TẠI (thời điểm xem)</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="7" t="n"/>
+      <c r="F23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="41" t="inlineStr">
         <is>
           <t>Chỉ số</t>
         </is>
       </c>
-      <c r="B8" s="27" t="inlineStr">
-        <is>
-          <t>Kết quả</t>
-        </is>
-      </c>
-      <c r="C8" s="26" t="inlineStr">
-        <is>
-          <t>Ghi chú</t>
-        </is>
-      </c>
-      <c r="D8" s="81" t="n"/>
-      <c r="E8" s="81" t="n"/>
-      <c r="F8" s="81" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="52" t="inlineStr">
-        <is>
-          <t>Công việc hoàn thành</t>
-        </is>
-      </c>
-      <c r="B9" s="32">
-        <f>COUNTIFS('z_CV'!$B:$B,"&gt;="&amp;$N$4,'z_CV'!$B:$B,"&lt;="&amp;$O$4,'z_CV'!$O:$O,"Hoàn thành")</f>
-        <v/>
-      </c>
-      <c r="C9" s="35" t="inlineStr">
-        <is>
-          <t>Nhật ký công việc theo ngày</t>
-        </is>
-      </c>
-      <c r="D9" s="62" t="n"/>
-      <c r="E9" s="62" t="n"/>
-      <c r="F9" s="62" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="49" t="inlineStr">
-        <is>
-          <t>Công việc đang tiến hành</t>
-        </is>
-      </c>
-      <c r="B10" s="37">
-        <f>COUNTIFS('z_CV'!$B:$B,"&gt;="&amp;$N$4,'z_CV'!$B:$B,"&lt;="&amp;$O$4,'z_CV'!$O:$O,"Đang làm")</f>
-        <v/>
-      </c>
-      <c r="C10" s="40" t="inlineStr"/>
-      <c r="D10" s="65" t="n"/>
-      <c r="E10" s="65" t="n"/>
-      <c r="F10" s="65" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="52" t="inlineStr">
-        <is>
-          <t>Lỗi phát hiện</t>
-        </is>
-      </c>
-      <c r="B11" s="32">
-        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4)</f>
-        <v/>
-      </c>
-      <c r="C11" s="35" t="inlineStr">
-        <is>
-          <t>Theo Ngày phát hiện (05_Lỗi_Tester)</t>
-        </is>
-      </c>
-      <c r="D11" s="62" t="n"/>
-      <c r="E11" s="62" t="n"/>
-      <c r="F11" s="62" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Critical</t>
-        </is>
-      </c>
-      <c r="B12" s="82">
+      <c r="B24" s="42" t="inlineStr">
+        <is>
+          <t>Số lượng</t>
+        </is>
+      </c>
+      <c r="C24" s="42" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="D24" s="42" t="inlineStr">
+        <is>
+          <t>Tỷ lệ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="19" customHeight="1">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>I. KIỂM TRA WEBSITE</t>
+        </is>
+      </c>
+      <c r="B25" s="29" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="29" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="inlineStr">
+        <is>
+          <t>Trang hoàn thành</t>
+        </is>
+      </c>
+      <c r="B26" s="44">
+        <f>'z_Trang'!$D$1</f>
+        <v/>
+      </c>
+      <c r="C26" s="45">
+        <f>'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D26" s="46">
+        <f>'z_Trang'!$F$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="47" t="inlineStr">
+        <is>
+          <t>Trang đang kiểm tra</t>
+        </is>
+      </c>
+      <c r="B27" s="37">
+        <f>'z_Trang'!$H$1</f>
+        <v/>
+      </c>
+      <c r="C27" s="48">
+        <f>'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D27" s="49">
+        <f>'z_Trang'!$H$1/'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="50" t="inlineStr">
+        <is>
+          <t>Trang cần kiểm tra lại</t>
+        </is>
+      </c>
+      <c r="B28" s="32">
+        <f>'z_Trang'!$J$1</f>
+        <v/>
+      </c>
+      <c r="C28" s="51">
+        <f>'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D28" s="52">
+        <f>'z_Trang'!$J$1/'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>Trang chưa kiểm tra</t>
+        </is>
+      </c>
+      <c r="B29" s="37">
+        <f>'z_Trang'!$L$1</f>
+        <v/>
+      </c>
+      <c r="C29" s="48">
+        <f>'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D29" s="49">
+        <f>'z_Trang'!$L$1/'z_Trang'!$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="43" t="inlineStr">
+        <is>
+          <t>Tính năng hoàn thành</t>
+        </is>
+      </c>
+      <c r="B30" s="44">
+        <f>'z_TinhNang'!$D$1</f>
+        <v/>
+      </c>
+      <c r="C30" s="45">
+        <f>'z_TinhNang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D30" s="46">
+        <f>'z_TinhNang'!$F$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="47" t="inlineStr">
+        <is>
+          <t>Tính năng cần kiểm tra lại</t>
+        </is>
+      </c>
+      <c r="B31" s="37">
+        <f>'z_TinhNang'!$J$1</f>
+        <v/>
+      </c>
+      <c r="C31" s="48">
+        <f>'z_TinhNang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D31" s="49">
+        <f>'z_TinhNang'!$J$1/'z_TinhNang'!$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="50" t="inlineStr">
+        <is>
+          <t>Tính năng chưa kiểm tra</t>
+        </is>
+      </c>
+      <c r="B32" s="32">
+        <f>'z_TinhNang'!$L$1</f>
+        <v/>
+      </c>
+      <c r="C32" s="51">
+        <f>'z_TinhNang'!$B$1</f>
+        <v/>
+      </c>
+      <c r="D32" s="52">
+        <f>'z_TinhNang'!$L$1/'z_TinhNang'!$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="47" t="inlineStr">
+        <is>
+          <t>Tổng lỗi ghi nhận</t>
+        </is>
+      </c>
+      <c r="B33" s="37">
+        <f>COUNTA('z_Loi'!$E:$E)-1</f>
+        <v/>
+      </c>
+      <c r="C33" s="53" t="n"/>
+      <c r="D33" s="39" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="54" t="inlineStr">
+        <is>
+          <t>Lỗi đang mở (Open + Chưa gửi Dev)</t>
+        </is>
+      </c>
+      <c r="B34" s="55">
+        <f>(COUNTIF('z_Loi'!$U:$U,"Open")+COUNTIF('z_Loi'!$U:$U,"Chưa gửi Dev"))</f>
+        <v/>
+      </c>
+      <c r="C34" s="56" t="n"/>
+      <c r="D34" s="57" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="54" t="inlineStr">
+        <is>
+          <t>Lỗi Critical/High đang mở</t>
+        </is>
+      </c>
+      <c r="B35" s="55">
+        <f>(COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"High")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"High"))</f>
+        <v/>
+      </c>
+      <c r="C35" s="56" t="n"/>
+      <c r="D35" s="57" t="n"/>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>II. DATABASE (tổng đã thêm)</t>
+        </is>
+      </c>
+      <c r="B36" s="29" t="n"/>
+      <c r="C36" s="29" t="n"/>
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="29" t="n"/>
+      <c r="F36" s="29" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="50" t="inlineStr">
+        <is>
+          <t>DB Doanh nghiệp</t>
+        </is>
+      </c>
+      <c r="B37" s="32">
+        <f>COUNTA('z_DB_DN'!$A:$A)</f>
+        <v/>
+      </c>
+      <c r="C37" s="58" t="n"/>
+      <c r="D37" s="34" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="47" t="inlineStr">
+        <is>
+          <t>DB HR</t>
+        </is>
+      </c>
+      <c r="B38" s="37">
+        <f>COUNTA('z_DB_HR'!$A:$A)</f>
+        <v/>
+      </c>
+      <c r="C38" s="53" t="n"/>
+      <c r="D38" s="39" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="50" t="inlineStr">
+        <is>
+          <t>DB Ứng viên</t>
+        </is>
+      </c>
+      <c r="B39" s="32">
+        <f>COUNTA('z_DB_UV'!$A:$A)</f>
+        <v/>
+      </c>
+      <c r="C39" s="58" t="n"/>
+      <c r="D39" s="34" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="47" t="inlineStr">
+        <is>
+          <t>Tin tuyển dụng đã đăng</t>
+        </is>
+      </c>
+      <c r="B40" s="37">
+        <f>COUNTA('z_DB_Tin'!$A:$A)</f>
+        <v/>
+      </c>
+      <c r="C40" s="53" t="n"/>
+      <c r="D40" s="39" t="n"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>TÌNH TRẠNG XỬ LÝ LỖI (toàn bộ)</t>
+        </is>
+      </c>
+      <c r="B42" s="7" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>Trạng thái</t>
+        </is>
+      </c>
+      <c r="B43" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+      <c r="C43" s="41" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="D43" s="59" t="n"/>
+      <c r="E43" s="59" t="n"/>
+      <c r="F43" s="59" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="60" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="B44" s="32">
+        <f>COUNTIF('z_Loi'!$U:$U,"Open")</f>
+        <v/>
+      </c>
+      <c r="C44" s="61" t="inlineStr">
+        <is>
+          <t>Lỗi đang mở, đã ghi nhận</t>
+        </is>
+      </c>
+      <c r="D44" s="62" t="n"/>
+      <c r="E44" s="62" t="n"/>
+      <c r="F44" s="62" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="63" t="inlineStr">
+        <is>
+          <t>Chưa gửi Dev</t>
+        </is>
+      </c>
+      <c r="B45" s="37">
+        <f>COUNTIF('z_Loi'!$U:$U,"Chưa gửi Dev")</f>
+        <v/>
+      </c>
+      <c r="C45" s="64" t="inlineStr">
+        <is>
+          <t>Chưa chuyển Dev xử lý</t>
+        </is>
+      </c>
+      <c r="D45" s="65" t="n"/>
+      <c r="E45" s="65" t="n"/>
+      <c r="F45" s="65" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="66" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="B46" s="32">
+        <f>COUNTIF('z_Loi'!$U:$U,"Fixed")</f>
+        <v/>
+      </c>
+      <c r="C46" s="61" t="inlineStr">
+        <is>
+          <t>Dev báo đã sửa</t>
+        </is>
+      </c>
+      <c r="D46" s="62" t="n"/>
+      <c r="E46" s="62" t="n"/>
+      <c r="F46" s="62" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="67" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="B47" s="37">
+        <f>COUNTIF('z_Loi'!$U:$U,"Verified")</f>
+        <v/>
+      </c>
+      <c r="C47" s="64" t="inlineStr">
+        <is>
+          <t>Đã retest đạt</t>
+        </is>
+      </c>
+      <c r="D47" s="65" t="n"/>
+      <c r="E47" s="65" t="n"/>
+      <c r="F47" s="65" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="68" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="B48" s="32">
+        <f>COUNTIF('z_Loi'!$U:$U,"Closed")</f>
+        <v/>
+      </c>
+      <c r="C48" s="61" t="inlineStr">
+        <is>
+          <t>Đã đóng</t>
+        </is>
+      </c>
+      <c r="D48" s="62" t="n"/>
+      <c r="E48" s="62" t="n"/>
+      <c r="F48" s="62" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="69" t="inlineStr">
+        <is>
+          <t>Deferred</t>
+        </is>
+      </c>
+      <c r="B49" s="37">
+        <f>COUNTIF('z_Loi'!$U:$U,"Deferred")</f>
+        <v/>
+      </c>
+      <c r="C49" s="64" t="inlineStr">
+        <is>
+          <t>Tạm hoãn / không sửa</t>
+        </is>
+      </c>
+      <c r="D49" s="65" t="n"/>
+      <c r="E49" s="65" t="n"/>
+      <c r="F49" s="65" t="n"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>PHÂN BỐ LỖI PHÁT HIỆN TRONG TUẦN</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="41" t="inlineStr">
+        <is>
+          <t>Theo mức độ</t>
+        </is>
+      </c>
+      <c r="B52" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+      <c r="D52" s="41" t="inlineStr">
+        <is>
+          <t>Theo thiết bị</t>
+        </is>
+      </c>
+      <c r="E52" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="60" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="B53" s="32">
         <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Critical")</f>
         <v/>
       </c>
-      <c r="C12" s="40" t="inlineStr"/>
-      <c r="D12" s="65" t="n"/>
-      <c r="E12" s="65" t="n"/>
-      <c r="F12" s="65" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    High</t>
-        </is>
-      </c>
-      <c r="B13" s="83">
+      <c r="D53" s="50" t="inlineStr">
+        <is>
+          <t>Desktop</t>
+        </is>
+      </c>
+      <c r="E53" s="32">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Desktop*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B54" s="37">
         <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"High")</f>
         <v/>
       </c>
-      <c r="C13" s="35" t="inlineStr"/>
-      <c r="D13" s="62" t="n"/>
-      <c r="E13" s="62" t="n"/>
-      <c r="F13" s="62" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Medium</t>
-        </is>
-      </c>
-      <c r="B14" s="84">
+      <c r="D54" s="47" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="E54" s="37">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Mobile*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="71" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="B55" s="32">
         <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Medium")</f>
         <v/>
       </c>
-      <c r="C14" s="40" t="inlineStr"/>
-      <c r="D14" s="65" t="n"/>
-      <c r="E14" s="65" t="n"/>
-      <c r="F14" s="65" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    Low</t>
-        </is>
-      </c>
-      <c r="B15" s="85">
+      <c r="D55" s="50" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="E55" s="32">
+        <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$M:$M,"*Tablet*")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="67" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B56" s="37">
         <f>COUNTIFS('z_Loi'!$Q:$Q,"&gt;="&amp;$N$4,'z_Loi'!$Q:$Q,"&lt;="&amp;$O$4,'z_Loi'!$L:$L,"Low")</f>
         <v/>
       </c>
-      <c r="C15" s="35" t="inlineStr"/>
-      <c r="D15" s="62" t="n"/>
-      <c r="E15" s="62" t="n"/>
-      <c r="F15" s="62" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="49" t="inlineStr">
-        <is>
-          <t>Lỗi còn mở hiện tại</t>
-        </is>
-      </c>
-      <c r="B16" s="82">
-        <f>(COUNTIF('z_Loi'!$U:$U,"Open")+COUNTIF('z_Loi'!$U:$U,"Chưa gửi Dev"))</f>
-        <v/>
-      </c>
-      <c r="C16" s="40" t="inlineStr">
-        <is>
-          <t>Open + Chưa gửi Dev (toàn bộ)</t>
-        </is>
-      </c>
-      <c r="D16" s="65" t="n"/>
-      <c r="E16" s="65" t="n"/>
-      <c r="F16" s="65" t="n"/>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>TIẾN ĐỘ TOÀN WEBSITE (thời điểm xem)</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="43" t="inlineStr">
-        <is>
-          <t>Chỉ số</t>
-        </is>
-      </c>
-      <c r="B19" s="44" t="inlineStr">
-        <is>
-          <t>Số lượng</t>
-        </is>
-      </c>
-      <c r="C19" s="44" t="inlineStr">
-        <is>
-          <t>Tỷ lệ</t>
-        </is>
-      </c>
-      <c r="D19" s="59" t="n"/>
-      <c r="E19" s="59" t="n"/>
-      <c r="F19" s="59" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="52" t="inlineStr">
-        <is>
-          <t>Trang hoàn thành</t>
-        </is>
-      </c>
-      <c r="B20" s="32">
-        <f>'z_Trang'!$D$1</f>
-        <v/>
-      </c>
-      <c r="C20" s="54">
-        <f>'z_Trang'!$F$1</f>
-        <v/>
-      </c>
-      <c r="D20" s="62" t="n"/>
-      <c r="E20" s="62" t="n"/>
-      <c r="F20" s="62" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="49" t="inlineStr">
-        <is>
-          <t>Tính năng hoàn thành</t>
-        </is>
-      </c>
-      <c r="B21" s="37">
-        <f>'z_TinhNang'!$D$1</f>
-        <v/>
-      </c>
-      <c r="C21" s="51">
-        <f>'z_TinhNang'!$F$1</f>
-        <v/>
-      </c>
-      <c r="D21" s="65" t="n"/>
-      <c r="E21" s="65" t="n"/>
-      <c r="F21" s="65" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="52" t="inlineStr">
-        <is>
-          <t>Trang cần kiểm tra lại</t>
-        </is>
-      </c>
-      <c r="B22" s="32">
-        <f>'z_Trang'!$J$1</f>
-        <v/>
-      </c>
-      <c r="C22" s="54">
-        <f>'z_Trang'!$J$1/'z_Trang'!$B$1</f>
-        <v/>
-      </c>
-      <c r="D22" s="62" t="n"/>
-      <c r="E22" s="62" t="n"/>
-      <c r="F22" s="62" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="49" t="inlineStr">
-        <is>
-          <t>Tính năng cần kiểm tra lại</t>
-        </is>
-      </c>
-      <c r="B23" s="37">
-        <f>'z_TinhNang'!$J$1</f>
-        <v/>
-      </c>
-      <c r="C23" s="51">
-        <f>'z_TinhNang'!$J$1/'z_TinhNang'!$B$1</f>
-        <v/>
-      </c>
-      <c r="D23" s="65" t="n"/>
-      <c r="E23" s="65" t="n"/>
-      <c r="F23" s="65" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="72" t="inlineStr">
+        <is>
+          <t>THANH TIẾN ĐỘ HOÀN THÀNH</t>
+        </is>
+      </c>
+      <c r="B58" s="59" t="n"/>
+      <c r="C58" s="59" t="n"/>
+      <c r="D58" s="59" t="n"/>
+      <c r="E58" s="59" t="n"/>
+      <c r="F58" s="59" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="73" t="inlineStr">
+        <is>
+          <t>Trang</t>
+        </is>
+      </c>
+      <c r="B59" s="74">
+        <f>REPT("█",ROUND('z_Trang'!$F$1*30,0))&amp;" "&amp;TEXT('z_Trang'!$F$1,"0.0%")</f>
+        <v/>
+      </c>
+      <c r="C59" s="62" t="n"/>
+      <c r="D59" s="62" t="n"/>
+      <c r="E59" s="62" t="n"/>
+      <c r="F59" s="62" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="75" t="inlineStr">
+        <is>
+          <t>Tính năng</t>
+        </is>
+      </c>
+      <c r="B60" s="76">
+        <f>REPT("█",ROUND('z_TinhNang'!$F$1*30,0))&amp;" "&amp;TEXT('z_TinhNang'!$F$1,"0.0%")</f>
+        <v/>
+      </c>
+      <c r="C60" s="65" t="n"/>
+      <c r="D60" s="65" t="n"/>
+      <c r="E60" s="65" t="n"/>
+      <c r="F60" s="65" t="n"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>CHI TIẾT: TRANG &amp; TÍNH NĂNG ĐÃ TEST TRONG TUẦN</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="7" t="n"/>
+      <c r="E62" s="7" t="n"/>
+      <c r="F62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="77" t="inlineStr">
+        <is>
+          <t>Liệt kê các trang/tính năng có Ngày test gần nhất trong kỳ (trạng thái Hoàn thành hoặc Kiểm tra lại).</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="n"/>
+      <c r="C63" s="5" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="5" t="n"/>
+      <c r="F63" s="5" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="41" t="inlineStr">
+        <is>
+          <t>TRANG đã test trong kỳ</t>
+        </is>
+      </c>
+      <c r="B64" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+      <c r="C64" s="42" t="inlineStr">
+        <is>
+          <t>Ngày test/retest</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="78">
+        <f>IFERROR(QUERY('z_TrangFull'!$A$1:$R$65,"select B, I, P where P &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and P &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' and (E = 'Hoàn thành' or E = 'Kiểm tra lại') order by P desc label B '', I '', P '' format P 'dd/mm/yyyy', I '#,##0'",1),"(không có trang test trong kỳ)")</f>
+        <v/>
+      </c>
+      <c r="B65" s="79" t="n"/>
+      <c r="C65" s="80" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="n"/>
+      <c r="B66" s="79" t="n"/>
+      <c r="C66" s="80" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="n"/>
+      <c r="B67" s="79" t="n"/>
+      <c r="C67" s="80" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="14" t="n"/>
+      <c r="B68" s="79" t="n"/>
+      <c r="C68" s="80" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="14" t="n"/>
+      <c r="B69" s="79" t="n"/>
+      <c r="C69" s="80" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="14" t="n"/>
+      <c r="B70" s="79" t="n"/>
+      <c r="C70" s="80" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="14" t="n"/>
+      <c r="B71" s="79" t="n"/>
+      <c r="C71" s="80" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="14" t="n"/>
+      <c r="B72" s="79" t="n"/>
+      <c r="C72" s="80" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="14" t="n"/>
+      <c r="B73" s="79" t="n"/>
+      <c r="C73" s="80" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="14" t="n"/>
+      <c r="B74" s="79" t="n"/>
+      <c r="C74" s="80" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="14" t="n"/>
+      <c r="B75" s="79" t="n"/>
+      <c r="C75" s="80" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="14" t="n"/>
+      <c r="B76" s="79" t="n"/>
+      <c r="C76" s="80" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="14" t="n"/>
+      <c r="B77" s="79" t="n"/>
+      <c r="C77" s="80" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="14" t="n"/>
+      <c r="B78" s="79" t="n"/>
+      <c r="C78" s="80" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="14" t="n"/>
+      <c r="B79" s="79" t="n"/>
+      <c r="C79" s="80" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="14" t="n"/>
+      <c r="B80" s="79" t="n"/>
+      <c r="C80" s="80" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n"/>
+      <c r="B81" s="79" t="n"/>
+      <c r="C81" s="80" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="n"/>
+      <c r="B82" s="79" t="n"/>
+      <c r="C82" s="80" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="n"/>
+      <c r="B83" s="79" t="n"/>
+      <c r="C83" s="80" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="14" t="n"/>
+      <c r="B84" s="79" t="n"/>
+      <c r="C84" s="80" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="14" t="n"/>
+      <c r="B85" s="79" t="n"/>
+      <c r="C85" s="80" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="14" t="n"/>
+      <c r="B86" s="79" t="n"/>
+      <c r="C86" s="80" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="14" t="n"/>
+      <c r="B87" s="79" t="n"/>
+      <c r="C87" s="80" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="14" t="n"/>
+      <c r="B88" s="79" t="n"/>
+      <c r="C88" s="80" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="14" t="n"/>
+      <c r="B89" s="79" t="n"/>
+      <c r="C89" s="80" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="14" t="n"/>
+      <c r="B90" s="79" t="n"/>
+      <c r="C90" s="80" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="14" t="n"/>
+      <c r="B91" s="79" t="n"/>
+      <c r="C91" s="80" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="14" t="n"/>
+      <c r="B92" s="79" t="n"/>
+      <c r="C92" s="80" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="14" t="n"/>
+      <c r="B93" s="79" t="n"/>
+      <c r="C93" s="80" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="14" t="n"/>
+      <c r="B94" s="79" t="n"/>
+      <c r="C94" s="80" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="14" t="n"/>
+      <c r="B95" s="79" t="n"/>
+      <c r="C95" s="80" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="14" t="n"/>
+      <c r="B96" s="79" t="n"/>
+      <c r="C96" s="80" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="14" t="n"/>
+      <c r="B97" s="79" t="n"/>
+      <c r="C97" s="80" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="14" t="n"/>
+      <c r="B98" s="79" t="n"/>
+      <c r="C98" s="80" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="14" t="n"/>
+      <c r="B99" s="79" t="n"/>
+      <c r="C99" s="80" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="n"/>
+      <c r="B100" s="79" t="n"/>
+      <c r="C100" s="80" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="n"/>
+      <c r="B101" s="79" t="n"/>
+      <c r="C101" s="80" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="n"/>
+      <c r="B102" s="79" t="n"/>
+      <c r="C102" s="80" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="n"/>
+      <c r="B103" s="79" t="n"/>
+      <c r="C103" s="80" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="n"/>
+      <c r="B104" s="79" t="n"/>
+      <c r="C104" s="80" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="n"/>
+      <c r="B105" s="79" t="n"/>
+      <c r="C105" s="80" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="n"/>
+      <c r="B106" s="79" t="n"/>
+      <c r="C106" s="80" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="n"/>
+      <c r="B107" s="79" t="n"/>
+      <c r="C107" s="80" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="n"/>
+      <c r="B108" s="79" t="n"/>
+      <c r="C108" s="80" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="n"/>
+      <c r="B109" s="79" t="n"/>
+      <c r="C109" s="80" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="n"/>
+      <c r="B110" s="79" t="n"/>
+      <c r="C110" s="80" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="14" t="n"/>
+      <c r="B111" s="79" t="n"/>
+      <c r="C111" s="80" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="n"/>
+      <c r="B112" s="79" t="n"/>
+      <c r="C112" s="80" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="14" t="n"/>
+      <c r="B113" s="79" t="n"/>
+      <c r="C113" s="80" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="n"/>
+      <c r="B114" s="79" t="n"/>
+      <c r="C114" s="80" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="14" t="n"/>
+      <c r="B115" s="79" t="n"/>
+      <c r="C115" s="80" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="n"/>
+      <c r="B116" s="79" t="n"/>
+      <c r="C116" s="80" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="14" t="n"/>
+      <c r="B117" s="79" t="n"/>
+      <c r="C117" s="80" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="n"/>
+      <c r="B118" s="79" t="n"/>
+      <c r="C118" s="80" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="14" t="n"/>
+      <c r="B119" s="79" t="n"/>
+      <c r="C119" s="80" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="n"/>
+      <c r="B120" s="79" t="n"/>
+      <c r="C120" s="80" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="14" t="n"/>
+      <c r="B121" s="79" t="n"/>
+      <c r="C121" s="80" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="n"/>
+      <c r="B122" s="79" t="n"/>
+      <c r="C122" s="80" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="14" t="n"/>
+      <c r="B123" s="79" t="n"/>
+      <c r="C123" s="80" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="n"/>
+      <c r="B124" s="79" t="n"/>
+      <c r="C124" s="80" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="14" t="n"/>
+      <c r="B125" s="79" t="n"/>
+      <c r="C125" s="80" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="n"/>
+      <c r="B126" s="79" t="n"/>
+      <c r="C126" s="80" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="14" t="n"/>
+      <c r="B127" s="79" t="n"/>
+      <c r="C127" s="80" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="n"/>
+      <c r="B128" s="79" t="n"/>
+      <c r="C128" s="80" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="41" t="inlineStr">
+        <is>
+          <t>TÍNH NĂNG đã test trong kỳ</t>
+        </is>
+      </c>
+      <c r="B130" s="42" t="inlineStr">
+        <is>
+          <t>Số lỗi</t>
+        </is>
+      </c>
+      <c r="C130" s="42" t="inlineStr">
+        <is>
+          <t>Ngày test/retest</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="78">
+        <f>IFERROR(QUERY('z_TNFull'!$A$1:$T$89,"select B, K, R where R &gt;= date '"&amp;TEXT($N$4,"yyyy-mm-dd")&amp;"' and R &lt;= date '"&amp;TEXT($O$4,"yyyy-mm-dd")&amp;"' and (J = 'Hoàn thành' or J = 'Kiểm tra lại') order by R desc label B '', K '', R '' format R 'dd/mm/yyyy', K '#,##0'",1),"(không có tính năng test trong kỳ)")</f>
+        <v/>
+      </c>
+      <c r="B131" s="79" t="n"/>
+      <c r="C131" s="80" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="n"/>
+      <c r="B132" s="79" t="n"/>
+      <c r="C132" s="80" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="14" t="n"/>
+      <c r="B133" s="79" t="n"/>
+      <c r="C133" s="80" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="14" t="n"/>
+      <c r="B134" s="79" t="n"/>
+      <c r="C134" s="80" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="14" t="n"/>
+      <c r="B135" s="79" t="n"/>
+      <c r="C135" s="80" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="14" t="n"/>
+      <c r="B136" s="79" t="n"/>
+      <c r="C136" s="80" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="14" t="n"/>
+      <c r="B137" s="79" t="n"/>
+      <c r="C137" s="80" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="n"/>
+      <c r="B138" s="79" t="n"/>
+      <c r="C138" s="80" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="14" t="n"/>
+      <c r="B139" s="79" t="n"/>
+      <c r="C139" s="80" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="14" t="n"/>
+      <c r="B140" s="79" t="n"/>
+      <c r="C140" s="80" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="14" t="n"/>
+      <c r="B141" s="79" t="n"/>
+      <c r="C141" s="80" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="14" t="n"/>
+      <c r="B142" s="79" t="n"/>
+      <c r="C142" s="80" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="14" t="n"/>
+      <c r="B143" s="79" t="n"/>
+      <c r="C143" s="80" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="14" t="n"/>
+      <c r="B144" s="79" t="n"/>
+      <c r="C144" s="80" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="14" t="n"/>
+      <c r="B145" s="79" t="n"/>
+      <c r="C145" s="80" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="14" t="n"/>
+      <c r="B146" s="79" t="n"/>
+      <c r="C146" s="80" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="14" t="n"/>
+      <c r="B147" s="79" t="n"/>
+      <c r="C147" s="80" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="14" t="n"/>
+      <c r="B148" s="79" t="n"/>
+      <c r="C148" s="80" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="14" t="n"/>
+      <c r="B149" s="79" t="n"/>
+      <c r="C149" s="80" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="14" t="n"/>
+      <c r="B150" s="79" t="n"/>
+      <c r="C150" s="80" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="14" t="n"/>
+      <c r="B151" s="79" t="n"/>
+      <c r="C151" s="80" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="14" t="n"/>
+      <c r="B152" s="79" t="n"/>
+      <c r="C152" s="80" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="14" t="n"/>
+      <c r="B153" s="79" t="n"/>
+      <c r="C153" s="80" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="14" t="n"/>
+      <c r="B154" s="79" t="n"/>
+      <c r="C154" s="80" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="14" t="n"/>
+      <c r="B155" s="79" t="n"/>
+      <c r="C155" s="80" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="14" t="n"/>
+      <c r="B156" s="79" t="n"/>
+      <c r="C156" s="80" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="14" t="n"/>
+      <c r="B157" s="79" t="n"/>
+      <c r="C157" s="80" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="14" t="n"/>
+      <c r="B158" s="79" t="n"/>
+      <c r="C158" s="80" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="14" t="n"/>
+      <c r="B159" s="79" t="n"/>
+      <c r="C159" s="80" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="14" t="n"/>
+      <c r="B160" s="79" t="n"/>
+      <c r="C160" s="80" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="14" t="n"/>
+      <c r="B161" s="79" t="n"/>
+      <c r="C161" s="80" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="14" t="n"/>
+      <c r="B162" s="79" t="n"/>
+      <c r="C162" s="80" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="14" t="n"/>
+      <c r="B163" s="79" t="n"/>
+      <c r="C163" s="80" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="14" t="n"/>
+      <c r="B164" s="79" t="n"/>
+      <c r="C164" s="80" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="14" t="n"/>
+      <c r="B165" s="79" t="n"/>
+      <c r="C165" s="80" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="14" t="n"/>
+      <c r="B166" s="79" t="n"/>
+      <c r="C166" s="80" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="14" t="n"/>
+      <c r="B167" s="79" t="n"/>
+      <c r="C167" s="80" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="14" t="n"/>
+      <c r="B168" s="79" t="n"/>
+      <c r="C168" s="80" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="14" t="n"/>
+      <c r="B169" s="79" t="n"/>
+      <c r="C169" s="80" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="14" t="n"/>
+      <c r="B170" s="79" t="n"/>
+      <c r="C170" s="80" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="14" t="n"/>
+      <c r="B171" s="79" t="n"/>
+      <c r="C171" s="80" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="14" t="n"/>
+      <c r="B172" s="79" t="n"/>
+      <c r="C172" s="80" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="14" t="n"/>
+      <c r="B173" s="79" t="n"/>
+      <c r="C173" s="80" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="14" t="n"/>
+      <c r="B174" s="79" t="n"/>
+      <c r="C174" s="80" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="14" t="n"/>
+      <c r="B175" s="79" t="n"/>
+      <c r="C175" s="80" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="14" t="n"/>
+      <c r="B176" s="79" t="n"/>
+      <c r="C176" s="80" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="14" t="n"/>
+      <c r="B177" s="79" t="n"/>
+      <c r="C177" s="80" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="14" t="n"/>
+      <c r="B178" s="79" t="n"/>
+      <c r="C178" s="80" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="14" t="n"/>
+      <c r="B179" s="79" t="n"/>
+      <c r="C179" s="80" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="14" t="n"/>
+      <c r="B180" s="79" t="n"/>
+      <c r="C180" s="80" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="14" t="n"/>
+      <c r="B181" s="79" t="n"/>
+      <c r="C181" s="80" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="14" t="n"/>
+      <c r="B182" s="79" t="n"/>
+      <c r="C182" s="80" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="14" t="n"/>
+      <c r="B183" s="79" t="n"/>
+      <c r="C183" s="80" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="14" t="n"/>
+      <c r="B184" s="79" t="n"/>
+      <c r="C184" s="80" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="14" t="n"/>
+      <c r="B185" s="79" t="n"/>
+      <c r="C185" s="80" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="14" t="n"/>
+      <c r="B186" s="79" t="n"/>
+      <c r="C186" s="80" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="14" t="n"/>
+      <c r="B187" s="79" t="n"/>
+      <c r="C187" s="80" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="14" t="n"/>
+      <c r="B188" s="79" t="n"/>
+      <c r="C188" s="80" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="14" t="n"/>
+      <c r="B189" s="79" t="n"/>
+      <c r="C189" s="80" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="14" t="n"/>
+      <c r="B190" s="79" t="n"/>
+      <c r="C190" s="80" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="14" t="n"/>
+      <c r="B191" s="79" t="n"/>
+      <c r="C191" s="80" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="14" t="n"/>
+      <c r="B192" s="79" t="n"/>
+      <c r="C192" s="80" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="14" t="n"/>
+      <c r="B193" s="79" t="n"/>
+      <c r="C193" s="80" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="14" t="n"/>
+      <c r="B194" s="79" t="n"/>
+      <c r="C194" s="80" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="14" t="n"/>
+      <c r="B195" s="79" t="n"/>
+      <c r="C195" s="80" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="14" t="n"/>
+      <c r="B196" s="79" t="n"/>
+      <c r="C196" s="80" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="14" t="n"/>
+      <c r="B197" s="79" t="n"/>
+      <c r="C197" s="80" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="14" t="n"/>
+      <c r="B198" s="79" t="n"/>
+      <c r="C198" s="80" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="14" t="n"/>
+      <c r="B199" s="79" t="n"/>
+      <c r="C199" s="80" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="14" t="n"/>
+      <c r="B200" s="79" t="n"/>
+      <c r="C200" s="80" t="n"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="14" t="n"/>
+      <c r="B201" s="79" t="n"/>
+      <c r="C201" s="80" t="n"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="14" t="n"/>
+      <c r="B202" s="79" t="n"/>
+      <c r="C202" s="80" t="n"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="14" t="n"/>
+      <c r="B203" s="79" t="n"/>
+      <c r="C203" s="80" t="n"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="14" t="n"/>
+      <c r="B204" s="79" t="n"/>
+      <c r="C204" s="80" t="n"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="14" t="n"/>
+      <c r="B205" s="79" t="n"/>
+      <c r="C205" s="80" t="n"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="14" t="n"/>
+      <c r="B206" s="79" t="n"/>
+      <c r="C206" s="80" t="n"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="14" t="n"/>
+      <c r="B207" s="79" t="n"/>
+      <c r="C207" s="80" t="n"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="14" t="n"/>
+      <c r="B208" s="79" t="n"/>
+      <c r="C208" s="80" t="n"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="14" t="n"/>
+      <c r="B209" s="79" t="n"/>
+      <c r="C209" s="80" t="n"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="14" t="n"/>
+      <c r="B210" s="79" t="n"/>
+      <c r="C210" s="80" t="n"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="14" t="n"/>
+      <c r="B211" s="79" t="n"/>
+      <c r="C211" s="80" t="n"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="14" t="n"/>
+      <c r="B212" s="79" t="n"/>
+      <c r="C212" s="80" t="n"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="14" t="n"/>
+      <c r="B213" s="79" t="n"/>
+      <c r="C213" s="80" t="n"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="14" t="n"/>
+      <c r="B214" s="79" t="n"/>
+      <c r="C214" s="80" t="n"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="14" t="n"/>
+      <c r="B215" s="79" t="n"/>
+      <c r="C215" s="80" t="n"/>
+    </row>
+    <row r="216">
+      <c r="A216" s="14" t="n"/>
+      <c r="B216" s="79" t="n"/>
+      <c r="C216" s="80" t="n"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="14" t="n"/>
+      <c r="B217" s="79" t="n"/>
+      <c r="C217" s="80" t="n"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="14" t="n"/>
+      <c r="B218" s="79" t="n"/>
+      <c r="C218" s="80" t="n"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="14" t="n"/>
+      <c r="B219" s="79" t="n"/>
+      <c r="C219" s="80" t="n"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="14" t="n"/>
+      <c r="B220" s="79" t="n"/>
+      <c r="C220" s="80" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="C13:F13"/>
+  <mergeCells count="23">
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="B59:F59"/>
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A62:F62"/>
+    <mergeCell ref="A63:F63"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="C44:F44"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A36:F36"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="D5:E5"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
@@ -2883,7 +5096,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="008B5E00"/>
@@ -2932,70 +5145,70 @@
       <c r="H2" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="A4" s="42" t="inlineStr">
         <is>
           <t>Kỳ nghiệm thu</t>
         </is>
       </c>
-      <c r="B4" s="86" t="inlineStr">
+      <c r="B4" s="85" t="inlineStr">
         <is>
           <t>Tháng 8</t>
         </is>
       </c>
-      <c r="C4" s="44" t="inlineStr">
+      <c r="C4" s="42" t="inlineStr">
         <is>
           <t>Ngày lập</t>
         </is>
       </c>
-      <c r="D4" s="87">
+      <c r="D4" s="86">
         <f>TODAY()</f>
         <v/>
       </c>
-      <c r="E4" s="88" t="n"/>
-      <c r="F4" s="44" t="inlineStr">
+      <c r="E4" s="87" t="n"/>
+      <c r="F4" s="42" t="inlineStr">
         <is>
           <t>Người lập</t>
         </is>
       </c>
-      <c r="G4" s="89" t="inlineStr"/>
+      <c r="G4" s="88" t="inlineStr"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="90" t="inlineStr">
+      <c r="A6" s="89" t="inlineStr">
         <is>
           <t>Hạng mục</t>
         </is>
       </c>
-      <c r="B6" s="90" t="inlineStr">
+      <c r="B6" s="89" t="inlineStr">
         <is>
           <t>Phạm vi</t>
         </is>
       </c>
-      <c r="C6" s="90" t="inlineStr">
+      <c r="C6" s="89" t="inlineStr">
         <is>
           <t>Tổng</t>
         </is>
       </c>
-      <c r="D6" s="90" t="inlineStr">
+      <c r="D6" s="89" t="inlineStr">
         <is>
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="E6" s="90" t="inlineStr">
+      <c r="E6" s="89" t="inlineStr">
         <is>
           <t>Tỷ lệ</t>
         </is>
       </c>
-      <c r="F6" s="90" t="inlineStr">
+      <c r="F6" s="89" t="inlineStr">
         <is>
           <t>Critical/High mở</t>
         </is>
       </c>
-      <c r="G6" s="90" t="inlineStr">
+      <c r="G6" s="89" t="inlineStr">
         <is>
           <t>Kết luận</t>
         </is>
       </c>
-      <c r="H6" s="90" t="inlineStr">
+      <c r="H6" s="89" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
@@ -3007,16 +5220,16 @@
           <t>UI/UX</t>
         </is>
       </c>
-      <c r="B7" s="91" t="inlineStr">
+      <c r="B7" s="90" t="inlineStr">
         <is>
           <t>Trang website</t>
         </is>
       </c>
-      <c r="C7" s="53">
+      <c r="C7" s="51">
         <f>'z_Trang'!$B$1</f>
         <v/>
       </c>
-      <c r="D7" s="92">
+      <c r="D7" s="91">
         <f>'z_Trang'!$D$1</f>
         <v/>
       </c>
@@ -3024,16 +5237,16 @@
         <f>'z_Trang'!$F$1</f>
         <v/>
       </c>
-      <c r="F7" s="93">
+      <c r="F7" s="92">
         <f>(COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"High")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"High"))</f>
         <v/>
       </c>
-      <c r="G7" s="94" t="inlineStr">
+      <c r="G7" s="93" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
       </c>
-      <c r="H7" s="77" t="inlineStr"/>
+      <c r="H7" s="78" t="inlineStr"/>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="75" t="inlineStr">
@@ -3041,16 +5254,16 @@
           <t>Chức năng</t>
         </is>
       </c>
-      <c r="B8" s="95" t="inlineStr">
+      <c r="B8" s="94" t="inlineStr">
         <is>
           <t>88 tính năng</t>
         </is>
       </c>
-      <c r="C8" s="50">
+      <c r="C8" s="48">
         <f>'z_TinhNang'!$B$1</f>
         <v/>
       </c>
-      <c r="D8" s="96">
+      <c r="D8" s="95">
         <f>'z_TinhNang'!$D$1</f>
         <v/>
       </c>
@@ -3058,16 +5271,16 @@
         <f>'z_TinhNang'!$F$1</f>
         <v/>
       </c>
-      <c r="F8" s="97">
+      <c r="F8" s="96">
         <f>(COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Open",'z_Loi'!$L:$L,"High")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"Critical")+COUNTIFS('z_Loi'!$U:$U,"Chưa gửi Dev",'z_Loi'!$L:$L,"High"))</f>
         <v/>
       </c>
-      <c r="G8" s="98" t="inlineStr">
+      <c r="G8" s="97" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
       </c>
-      <c r="H8" s="99" t="inlineStr"/>
+      <c r="H8" s="98" t="inlineStr"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="73" t="inlineStr">
@@ -3075,24 +5288,24 @@
           <t>Responsive</t>
         </is>
       </c>
-      <c r="B9" s="91" t="inlineStr">
+      <c r="B9" s="90" t="inlineStr">
         <is>
           <t>YC_87 + lỗi responsive</t>
         </is>
       </c>
-      <c r="C9" s="53" t="inlineStr"/>
-      <c r="D9" s="92" t="inlineStr"/>
-      <c r="E9" s="41" t="inlineStr"/>
-      <c r="F9" s="93">
+      <c r="C9" s="51" t="inlineStr"/>
+      <c r="D9" s="91" t="inlineStr"/>
+      <c r="E9" s="58" t="inlineStr"/>
+      <c r="F9" s="92">
         <f>COUNTIF('z_Loi'!$K:$K,"*Responsive*")</f>
         <v/>
       </c>
-      <c r="G9" s="94" t="inlineStr">
+      <c r="G9" s="93" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
       </c>
-      <c r="H9" s="77" t="inlineStr"/>
+      <c r="H9" s="78" t="inlineStr"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="75" t="inlineStr">
@@ -3100,24 +5313,24 @@
           <t>Bảo mật</t>
         </is>
       </c>
-      <c r="B10" s="95" t="inlineStr">
+      <c r="B10" s="94" t="inlineStr">
         <is>
           <t>Test Case Security</t>
         </is>
       </c>
-      <c r="C10" s="50" t="inlineStr"/>
-      <c r="D10" s="96" t="inlineStr"/>
-      <c r="E10" s="42" t="inlineStr"/>
-      <c r="F10" s="97">
+      <c r="C10" s="48" t="inlineStr"/>
+      <c r="D10" s="95" t="inlineStr"/>
+      <c r="E10" s="53" t="inlineStr"/>
+      <c r="F10" s="96">
         <f>COUNTIF('z_Loi'!$K:$K,"*Security*")</f>
         <v/>
       </c>
-      <c r="G10" s="98" t="inlineStr">
+      <c r="G10" s="97" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
       </c>
-      <c r="H10" s="99" t="inlineStr"/>
+      <c r="H10" s="98" t="inlineStr"/>
     </row>
     <row r="11" ht="26" customHeight="1">
       <c r="A11" s="73" t="inlineStr">
@@ -3125,21 +5338,21 @@
           <t>Dữ liệu</t>
         </is>
       </c>
-      <c r="B11" s="91" t="inlineStr">
+      <c r="B11" s="90" t="inlineStr">
         <is>
           <t>Test Case API/Database</t>
         </is>
       </c>
-      <c r="C11" s="53" t="inlineStr"/>
-      <c r="D11" s="92" t="inlineStr"/>
-      <c r="E11" s="41" t="inlineStr"/>
-      <c r="F11" s="100" t="inlineStr"/>
-      <c r="G11" s="94" t="inlineStr">
+      <c r="C11" s="51" t="inlineStr"/>
+      <c r="D11" s="91" t="inlineStr"/>
+      <c r="E11" s="58" t="inlineStr"/>
+      <c r="F11" s="99" t="inlineStr"/>
+      <c r="G11" s="93" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
       </c>
-      <c r="H11" s="77" t="inlineStr"/>
+      <c r="H11" s="78" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="72" t="inlineStr">
@@ -3148,7 +5361,7 @@
         </is>
       </c>
       <c r="B13" s="59" t="n"/>
-      <c r="C13" s="101" t="inlineStr">
+      <c r="C13" s="100" t="inlineStr">
         <is>
           <t>Chưa nghiệm thu</t>
         </is>
@@ -3160,18 +5373,18 @@
       <c r="H13" s="62" t="n"/>
     </row>
     <row r="14" ht="34" customHeight="1">
-      <c r="A14" s="102" t="inlineStr">
+      <c r="A14" s="101" t="inlineStr">
         <is>
           <t>Điều kiện khuyến nghị: không còn Critical/High chưa được phê duyệt; phạm vi và bằng chứng đầy đủ; ngoại lệ phải có người duyệt và lý do rõ ràng.</t>
         </is>
       </c>
-      <c r="B14" s="103" t="n"/>
-      <c r="C14" s="103" t="n"/>
-      <c r="D14" s="103" t="n"/>
-      <c r="E14" s="103" t="n"/>
-      <c r="F14" s="103" t="n"/>
-      <c r="G14" s="103" t="n"/>
-      <c r="H14" s="103" t="n"/>
+      <c r="B14" s="102" t="n"/>
+      <c r="C14" s="102" t="n"/>
+      <c r="D14" s="102" t="n"/>
+      <c r="E14" s="102" t="n"/>
+      <c r="F14" s="102" t="n"/>
+      <c r="G14" s="102" t="n"/>
+      <c r="H14" s="102" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -3237,7 +5450,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$1,"05_Lỗi_Tester!A4:V606")</f>
+        <f>IMPORTRANGE('z_Config'!$B$1,"02_UI_UX!A4:R68")</f>
         <v/>
       </c>
     </row>
@@ -3257,7 +5470,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$1,"01_Cong_viec_ngay!A4:P1004")</f>
+        <f>IMPORTRANGE('z_Config'!$B$1,"03_Tính_năng!A4:T92")</f>
         <v/>
       </c>
     </row>
@@ -3277,7 +5490,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$3,"'HS DN'!D4:N970")</f>
+        <f>IMPORTRANGE('z_Config'!$B$1,"05_Lỗi_Tester!A4:V606")</f>
         <v/>
       </c>
     </row>
@@ -3297,7 +5510,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$3,"'HS HR'!D4:E966")</f>
+        <f>IMPORTRANGE('z_Config'!$B$1,"01_Cong_viec_ngay!A4:P1004")</f>
         <v/>
       </c>
     </row>
@@ -3317,7 +5530,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$3,"'HS ỨNG TUYỂN'!D5:D990")</f>
+        <f>IMPORTRANGE('z_Config'!$B$3,"'HS DN'!D4:N970")</f>
         <v/>
       </c>
     </row>
@@ -3337,7 +5550,7 @@
   <sheetData>
     <row r="1">
       <c r="A1">
-        <f>IMPORTRANGE('z_Config'!$B$3,"'Tin tuyển dụng'!C4:D1006")</f>
+        <f>IMPORTRANGE('z_Config'!$B$3,"'HS HR'!D4:E966")</f>
         <v/>
       </c>
     </row>

</xml_diff>